<commit_message>
finanze: semplifica il foglio Movimenti, niente più SUMIFS
Rimosso il riepilogo automatico per categoria/settimana: era troppo
rigido da estendere a mano. Il foglio ora è solo una tabella piatta
(Data, Descrizione, Importo, Categoria) senza formule, così aggiungere
una categoria nuova è solo scrivere del testo. Corrette anche le due
voci lasciate "da verificare": erano benzina, e Scotti Andrea è cibo
(carne, Cascina de Lassi a Landriano).
</commit_message>
<xml_diff>
--- a/finanze/quaderno-5000.xlsx
+++ b/finanze/quaderno-5000.xlsx
@@ -21,12 +21,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="#,##0&quot; €&quot;;(#,##0)&quot; €&quot;;&quot;–&quot;"/>
-    <numFmt numFmtId="167" formatCode="&quot;Sett. dal&quot; dd/mm"/>
-    <numFmt numFmtId="168" formatCode="#,##0.00&quot; €&quot;;(#,##0.00)&quot; €&quot;;&quot;–&quot;"/>
+    <numFmt numFmtId="167" formatCode="#,##0.00&quot; €&quot;;(#,##0.00)&quot; €&quot;;&quot;–&quot;"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -110,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -139,12 +138,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -7037,404 +7032,455 @@
   <dimension ref="A1:D300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="58" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Movimenti PostePay + buoni pasto — spese per categoria</t>
+          <t>Movimenti PostePay + buoni pasto — dati grezzi</t>
         </is>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Ogni settimana (o ogni mese, come preferisci) esporta i movimenti da PostePay e incollali qui sotto; le due colonne EdenRed dei buoni pasto vanno aggiunte a mano. La categoria la scrivo io leggendo la descrizione. Il riepilogo qui sopra si aggiorna da solo.</t>
+          <t>Nessuna formula qui dentro: è solo un elenco. Le somme e i confronti li fai tu, come vuoi. Per aggiungere una categoria nuova basta scriverla nella colonna Categoria — non c'è nulla da rompere. Il raggruppamento per data e categoria te lo preparo io in chat ogni volta che incolli i movimenti nuovi: tu li copi qui sotto così come sono.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Riepilogo per categoria e settimana</t>
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>Descrizione</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>Importo (€)</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>Categoria</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
-        <is>
-          <t>Categoria</t>
-        </is>
-      </c>
-      <c r="B5" s="22" t="n">
+      <c r="A5" s="15" t="n">
         <v>46272</v>
       </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>PostePay — ricarica per attivazione nuova carta (saldo trasferito dalla vecchia)</t>
+        </is>
+      </c>
       <c r="C5" s="22" t="n">
+        <v>980.1</v>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
+        <is>
+          <t>Trasferimento</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>EdenRed — ricarica 21 buoni pasto</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>189</v>
+      </c>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>Entrata</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>PostePay — POS 46084 San Donato (benzina)</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="n">
+        <v>-26.3</v>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>Benzina</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>PostePay — POS Market San Donato</t>
+        </is>
+      </c>
+      <c r="C8" s="22" t="n">
+        <v>-4.14</v>
+      </c>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>Cibo</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>PostePay — POS Ipercoop Peschiera Borromeo</t>
+        </is>
+      </c>
+      <c r="C9" s="22" t="n">
+        <v>-7.57</v>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>Cibo</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>PostePay — POS Scotti Andrea, Mediglia (Cascina de Lassi, Landriano — carne)</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="n">
+        <v>-46</v>
+      </c>
+      <c r="D10" s="17" t="inlineStr">
+        <is>
+          <t>Cibo</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>PostePay — commissioni PagoPA</t>
+        </is>
+      </c>
+      <c r="C11" s="22" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>Bollette</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>PostePay — avviso PagoPA, Ente 06655971007</t>
+        </is>
+      </c>
+      <c r="C12" s="22" t="n">
+        <v>-137.49</v>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>Bollette</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="n">
         <v>46279</v>
       </c>
-      <c r="D5" s="20" t="inlineStr">
-        <is>
-          <t>Totale</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>PostePay — commissioni PagoPA</t>
+        </is>
+      </c>
+      <c r="C13" s="22" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>Bollette</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>PostePay — avviso PagoPA, Ente 06655971007</t>
+        </is>
+      </c>
+      <c r="C14" s="22" t="n">
+        <v>-84.76000000000001</v>
+      </c>
+      <c r="D14" s="17" t="inlineStr">
+        <is>
+          <t>Bollette</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>PostePay — POS Esselunga San Giuliano Milanese</t>
+        </is>
+      </c>
+      <c r="C15" s="22" t="n">
+        <v>-1.95</v>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
         <is>
           <t>Cibo</t>
         </is>
       </c>
-      <c r="B6" s="23">
-        <f>SUMIFS($C$17:$C$300,$A$17:$A$300,"&gt;="&amp;B$5,$A$17:$A$300,"&lt;="&amp;(B$5+6),$D$17:$D$300,$A6)</f>
-        <v/>
-      </c>
-      <c r="C6" s="23">
-        <f>SUMIFS($C$17:$C$300,$A$17:$A$300,"&gt;="&amp;C$5,$A$17:$A$300,"&lt;="&amp;(C$5+6),$D$17:$D$300,$A6)</f>
-        <v/>
-      </c>
-      <c r="D6" s="24">
-        <f>SUM(B6:C6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="17" t="inlineStr">
-        <is>
-          <t>Bollette</t>
-        </is>
-      </c>
-      <c r="B7" s="23">
-        <f>SUMIFS($C$17:$C$300,$A$17:$A$300,"&gt;="&amp;B$5,$A$17:$A$300,"&lt;="&amp;(B$5+6),$D$17:$D$300,$A7)</f>
-        <v/>
-      </c>
-      <c r="C7" s="23">
-        <f>SUMIFS($C$17:$C$300,$A$17:$A$300,"&gt;="&amp;C$5,$A$17:$A$300,"&lt;="&amp;(C$5+6),$D$17:$D$300,$A7)</f>
-        <v/>
-      </c>
-      <c r="D7" s="24">
-        <f>SUM(B7:C7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="17" t="inlineStr">
-        <is>
-          <t>Abbonamenti</t>
-        </is>
-      </c>
-      <c r="B8" s="23">
-        <f>SUMIFS($C$17:$C$300,$A$17:$A$300,"&gt;="&amp;B$5,$A$17:$A$300,"&lt;="&amp;(B$5+6),$D$17:$D$300,$A8)</f>
-        <v/>
-      </c>
-      <c r="C8" s="23">
-        <f>SUMIFS($C$17:$C$300,$A$17:$A$300,"&gt;="&amp;C$5,$A$17:$A$300,"&lt;="&amp;(C$5+6),$D$17:$D$300,$A8)</f>
-        <v/>
-      </c>
-      <c r="D8" s="24">
-        <f>SUM(B8:C8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="17" t="inlineStr">
-        <is>
-          <t>Da verificare</t>
-        </is>
-      </c>
-      <c r="B9" s="23">
-        <f>SUMIFS($C$17:$C$300,$A$17:$A$300,"&gt;="&amp;B$5,$A$17:$A$300,"&lt;="&amp;(B$5+6),$D$17:$D$300,$A9)</f>
-        <v/>
-      </c>
-      <c r="C9" s="23">
-        <f>SUMIFS($C$17:$C$300,$A$17:$A$300,"&gt;="&amp;C$5,$A$17:$A$300,"&lt;="&amp;(C$5+6),$D$17:$D$300,$A9)</f>
-        <v/>
-      </c>
-      <c r="D9" s="24">
-        <f>SUM(B9:C9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Totale spese reali (esclude entrate e trasferimenti)</t>
-        </is>
-      </c>
-      <c r="B10" s="24">
-        <f>SUM(B6:B9)</f>
-        <v/>
-      </c>
-      <c r="C10" s="24">
-        <f>SUM(C6:C9)</f>
-        <v/>
-      </c>
-      <c r="D10" s="24">
-        <f>SUM(D6:D9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Entrata (informativo, escluso dal totale)</t>
-        </is>
-      </c>
-      <c r="B12" s="25">
-        <f>SUMIFS($C$17:$C$300,$A$17:$A$300,"&gt;="&amp;B$5,$A$17:$A$300,"&lt;="&amp;(B$5+6),$D$17:$D$300,"Entrata")</f>
-        <v/>
-      </c>
-      <c r="C12" s="25">
-        <f>SUMIFS($C$17:$C$300,$A$17:$A$300,"&gt;="&amp;C$5,$A$17:$A$300,"&lt;="&amp;(C$5+6),$D$17:$D$300,"Entrata")</f>
-        <v/>
-      </c>
-      <c r="D12" s="25">
-        <f>SUM(B12:C12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Trasferimento (informativo, escluso dal totale)</t>
-        </is>
-      </c>
-      <c r="B13" s="25">
-        <f>SUMIFS($C$17:$C$300,$A$17:$A$300,"&gt;="&amp;B$5,$A$17:$A$300,"&lt;="&amp;(B$5+6),$D$17:$D$300,"Trasferimento")</f>
-        <v/>
-      </c>
-      <c r="C13" s="25">
-        <f>SUMIFS($C$17:$C$300,$A$17:$A$300,"&gt;="&amp;C$5,$A$17:$A$300,"&lt;="&amp;(C$5+6),$D$17:$D$300,"Trasferimento")</f>
-        <v/>
-      </c>
-      <c r="D13" s="25">
-        <f>SUM(B13:C13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Movimenti dettagliati</t>
-        </is>
-      </c>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="inlineStr">
-        <is>
-          <t>Data</t>
-        </is>
-      </c>
-      <c r="B16" s="20" t="inlineStr">
-        <is>
-          <t>Descrizione</t>
-        </is>
-      </c>
-      <c r="C16" s="20" t="inlineStr">
-        <is>
-          <t>Importo (€)</t>
-        </is>
-      </c>
-      <c r="D16" s="20" t="inlineStr">
-        <is>
-          <t>Categoria</t>
+      <c r="A16" s="15" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>EdenRed — Essselunga (buono pasto)</t>
+        </is>
+      </c>
+      <c r="C16" s="22" t="n">
+        <v>-9</v>
+      </c>
+      <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t>Cibo</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="15" t="n">
-        <v>46272</v>
+        <v>46279</v>
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>PostePay — ricarica per attivazione nuova carta (saldo trasferito dalla vecchia)</t>
-        </is>
-      </c>
-      <c r="C17" s="26" t="n">
-        <v>980.1</v>
+          <t>EdenRed — Essselunga (2 buoni pasto)</t>
+        </is>
+      </c>
+      <c r="C17" s="22" t="n">
+        <v>-18</v>
       </c>
       <c r="D17" s="17" t="inlineStr">
         <is>
-          <t>Trasferimento</t>
+          <t>Cibo</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="n">
-        <v>46272</v>
+        <v>46280</v>
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>EdenRed — ricarica 21 buoni pasto</t>
-        </is>
-      </c>
-      <c r="C18" s="26" t="n">
-        <v>189</v>
+          <t>EdenRed — Meriggi (buono pasto)</t>
+        </is>
+      </c>
+      <c r="C18" s="22" t="n">
+        <v>-9</v>
       </c>
       <c r="D18" s="17" t="inlineStr">
         <is>
-          <t>Entrata</t>
+          <t>Cibo</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="n">
-        <v>46275</v>
+        <v>46280</v>
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>PostePay — POS 46084 San Donato (esercizio non identificato)</t>
-        </is>
-      </c>
-      <c r="C19" s="26" t="n">
-        <v>-26.3</v>
+          <t>PostePay — versamento sul Salvadanaio</t>
+        </is>
+      </c>
+      <c r="C19" s="22" t="n">
+        <v>-470</v>
       </c>
       <c r="D19" s="17" t="inlineStr">
         <is>
-          <t>Da verificare</t>
+          <t>Trasferimento</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="15" t="n">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>PostePay — POS Market San Donato</t>
-        </is>
-      </c>
-      <c r="C20" s="26" t="n">
-        <v>-4.14</v>
+          <t>PostePay — commissioni bonifico, estinzione conto BCC Caravaggio</t>
+        </is>
+      </c>
+      <c r="C20" s="22" t="n">
+        <v>-1</v>
       </c>
       <c r="D20" s="17" t="inlineStr">
         <is>
-          <t>Cibo</t>
+          <t>Trasferimento</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="15" t="n">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>PostePay — POS Ipercoop Peschiera Borromeo</t>
-        </is>
-      </c>
-      <c r="C21" s="26" t="n">
-        <v>-7.57</v>
+          <t>PostePay — bonifico SEPA istantaneo, estinzione conto BCC Caravaggio</t>
+        </is>
+      </c>
+      <c r="C21" s="22" t="n">
+        <v>-25</v>
       </c>
       <c r="D21" s="17" t="inlineStr">
         <is>
-          <t>Cibo</t>
+          <t>Trasferimento</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="15" t="n">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="B22" s="17" t="inlineStr">
         <is>
-          <t>PostePay — POS Scotti Andrea, Mediglia (non identificato)</t>
-        </is>
-      </c>
-      <c r="C22" s="26" t="n">
-        <v>-46</v>
+          <t>PostePay — POS PV1375, Milano (benzina)</t>
+        </is>
+      </c>
+      <c r="C22" s="22" t="n">
+        <v>-27.84</v>
       </c>
       <c r="D22" s="17" t="inlineStr">
         <is>
-          <t>Da verificare</t>
+          <t>Benzina</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="15" t="n">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>PostePay — commissioni PagoPA</t>
-        </is>
-      </c>
-      <c r="C23" s="26" t="n">
-        <v>-1.5</v>
+          <t>PostePay — POS Esselunga Monza</t>
+        </is>
+      </c>
+      <c r="C23" s="22" t="n">
+        <v>-1.73</v>
       </c>
       <c r="D23" s="17" t="inlineStr">
         <is>
-          <t>Bollette</t>
+          <t>Cibo</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="15" t="n">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>PostePay — avviso PagoPA, Ente 06655971007</t>
-        </is>
-      </c>
-      <c r="C24" s="26" t="n">
-        <v>-137.49</v>
+          <t>EdenRed — Esselunga (buono pasto)</t>
+        </is>
+      </c>
+      <c r="C24" s="22" t="n">
+        <v>-9</v>
       </c>
       <c r="D24" s="17" t="inlineStr">
         <is>
-          <t>Bollette</t>
+          <t>Cibo</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="15" t="n">
-        <v>46279</v>
+        <v>46281</v>
       </c>
       <c r="B25" s="17" t="inlineStr">
         <is>
-          <t>PostePay — commissioni PagoPA</t>
-        </is>
-      </c>
-      <c r="C25" s="26" t="n">
-        <v>-1.5</v>
+          <t>Anthropic — abbonamento Claude</t>
+        </is>
+      </c>
+      <c r="C25" s="22" t="n">
+        <v>-21.96</v>
       </c>
       <c r="D25" s="17" t="inlineStr">
         <is>
-          <t>Bollette</t>
+          <t>Abbonamenti</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="15" t="n">
-        <v>46279</v>
+        <v>46282</v>
       </c>
       <c r="B26" s="17" t="inlineStr">
         <is>
-          <t>PostePay — avviso PagoPA, Ente 06655971007</t>
-        </is>
-      </c>
-      <c r="C26" s="26" t="n">
-        <v>-84.76000000000001</v>
+          <t>PostePay — bonifico SEPA, residuo estinzione conto BCC Caravaggio</t>
+        </is>
+      </c>
+      <c r="C26" s="22" t="n">
+        <v>0.01</v>
       </c>
       <c r="D26" s="17" t="inlineStr">
         <is>
-          <t>Bollette</t>
+          <t>Trasferimento</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="15" t="n">
-        <v>46279</v>
+        <v>46284</v>
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>PostePay — POS Esselunga San Giuliano Milanese</t>
-        </is>
-      </c>
-      <c r="C27" s="26" t="n">
-        <v>-1.95</v>
+          <t>EdenRed — Tigros (3 buoni pasto)</t>
+        </is>
+      </c>
+      <c r="C27" s="22" t="n">
+        <v>-27</v>
       </c>
       <c r="D27" s="17" t="inlineStr">
         <is>
@@ -7444,15 +7490,15 @@
     </row>
     <row r="28">
       <c r="A28" s="15" t="n">
-        <v>46279</v>
+        <v>46284</v>
       </c>
       <c r="B28" s="17" t="inlineStr">
         <is>
-          <t>EdenRed — Essselunga (buono pasto)</t>
-        </is>
-      </c>
-      <c r="C28" s="26" t="n">
-        <v>-9</v>
+          <t>EdenRed — 2 movimenti non dettagliati (4 buoni pasto)</t>
+        </is>
+      </c>
+      <c r="C28" s="22" t="n">
+        <v>-36</v>
       </c>
       <c r="D28" s="17" t="inlineStr">
         <is>
@@ -7461,1790 +7507,1646 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="n">
-        <v>46279</v>
-      </c>
-      <c r="B29" s="17" t="inlineStr">
-        <is>
-          <t>EdenRed — Essselunga (2 buoni pasto)</t>
-        </is>
-      </c>
-      <c r="C29" s="26" t="n">
-        <v>-18</v>
-      </c>
-      <c r="D29" s="17" t="inlineStr">
-        <is>
-          <t>Cibo</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="15" t="n">
-        <v>46280</v>
-      </c>
-      <c r="B30" s="17" t="inlineStr">
-        <is>
-          <t>EdenRed — Meriggi (buono pasto)</t>
-        </is>
-      </c>
-      <c r="C30" s="26" t="n">
-        <v>-9</v>
-      </c>
-      <c r="D30" s="17" t="inlineStr">
-        <is>
-          <t>Cibo</t>
+      <c r="A29" s="18" t="n"/>
+      <c r="B29" s="19" t="n"/>
+      <c r="C29" s="23" t="n"/>
+      <c r="D29" s="19" t="n"/>
+    </row>
+    <row r="30" ht="50" customHeight="1">
+      <c r="A30" s="24" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>«Trasferimento» = spostamenti fra tuoi conti/chiusura BCC Caravaggio: non sono spesa reale, tienile fuori dai tuoi conteggi di spesa. Le 4 ricariche buoni pasto del 19/09 non erano nello screenshot: importo dedotto da 21 caricati − 9 rimasti − gli 8 già visti = 4.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="15" t="n">
-        <v>46280</v>
-      </c>
-      <c r="B31" s="17" t="inlineStr">
-        <is>
-          <t>PostePay — versamento sul Salvadanaio</t>
-        </is>
-      </c>
-      <c r="C31" s="26" t="n">
-        <v>-470</v>
-      </c>
-      <c r="D31" s="17" t="inlineStr">
-        <is>
-          <t>Trasferimento</t>
-        </is>
-      </c>
+      <c r="A31" s="18" t="n"/>
+      <c r="B31" s="19" t="n"/>
+      <c r="C31" s="23" t="n"/>
+      <c r="D31" s="19" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="15" t="n">
-        <v>46280</v>
-      </c>
-      <c r="B32" s="17" t="inlineStr">
-        <is>
-          <t>PostePay — commissioni bonifico, estinzione conto BCC Caravaggio</t>
-        </is>
-      </c>
-      <c r="C32" s="26" t="n">
-        <v>-1</v>
-      </c>
-      <c r="D32" s="17" t="inlineStr">
-        <is>
-          <t>Trasferimento</t>
-        </is>
-      </c>
+      <c r="A32" s="18" t="n"/>
+      <c r="B32" s="19" t="n"/>
+      <c r="C32" s="23" t="n"/>
+      <c r="D32" s="19" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="15" t="n">
-        <v>46280</v>
-      </c>
-      <c r="B33" s="17" t="inlineStr">
-        <is>
-          <t>PostePay — bonifico SEPA istantaneo, estinzione conto BCC Caravaggio</t>
-        </is>
-      </c>
-      <c r="C33" s="26" t="n">
-        <v>-25</v>
-      </c>
-      <c r="D33" s="17" t="inlineStr">
-        <is>
-          <t>Trasferimento</t>
-        </is>
-      </c>
+      <c r="A33" s="18" t="n"/>
+      <c r="B33" s="19" t="n"/>
+      <c r="C33" s="23" t="n"/>
+      <c r="D33" s="19" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="15" t="n">
-        <v>46281</v>
-      </c>
-      <c r="B34" s="17" t="inlineStr">
-        <is>
-          <t>PostePay — POS PV1375, Milano (non identificato)</t>
-        </is>
-      </c>
-      <c r="C34" s="26" t="n">
-        <v>-27.84</v>
-      </c>
-      <c r="D34" s="17" t="inlineStr">
-        <is>
-          <t>Da verificare</t>
-        </is>
-      </c>
+      <c r="A34" s="18" t="n"/>
+      <c r="B34" s="19" t="n"/>
+      <c r="C34" s="23" t="n"/>
+      <c r="D34" s="19" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="15" t="n">
-        <v>46281</v>
-      </c>
-      <c r="B35" s="17" t="inlineStr">
-        <is>
-          <t>PostePay — POS Esselunga Monza</t>
-        </is>
-      </c>
-      <c r="C35" s="26" t="n">
-        <v>-1.73</v>
-      </c>
-      <c r="D35" s="17" t="inlineStr">
-        <is>
-          <t>Cibo</t>
-        </is>
-      </c>
+      <c r="A35" s="18" t="n"/>
+      <c r="B35" s="19" t="n"/>
+      <c r="C35" s="23" t="n"/>
+      <c r="D35" s="19" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="15" t="n">
-        <v>46281</v>
-      </c>
-      <c r="B36" s="17" t="inlineStr">
-        <is>
-          <t>EdenRed — Esselunga (buono pasto)</t>
-        </is>
-      </c>
-      <c r="C36" s="26" t="n">
-        <v>-9</v>
-      </c>
-      <c r="D36" s="17" t="inlineStr">
-        <is>
-          <t>Cibo</t>
-        </is>
-      </c>
+      <c r="A36" s="18" t="n"/>
+      <c r="B36" s="19" t="n"/>
+      <c r="C36" s="23" t="n"/>
+      <c r="D36" s="19" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="15" t="n">
-        <v>46281</v>
-      </c>
-      <c r="B37" s="17" t="inlineStr">
-        <is>
-          <t>Anthropic — abbonamento Claude</t>
-        </is>
-      </c>
-      <c r="C37" s="26" t="n">
-        <v>-21.96</v>
-      </c>
-      <c r="D37" s="17" t="inlineStr">
-        <is>
-          <t>Abbonamenti</t>
-        </is>
-      </c>
+      <c r="A37" s="18" t="n"/>
+      <c r="B37" s="19" t="n"/>
+      <c r="C37" s="23" t="n"/>
+      <c r="D37" s="19" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="15" t="n">
-        <v>46282</v>
-      </c>
-      <c r="B38" s="17" t="inlineStr">
-        <is>
-          <t>PostePay — bonifico SEPA, residuo estinzione conto BCC Caravaggio</t>
-        </is>
-      </c>
-      <c r="C38" s="26" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="D38" s="17" t="inlineStr">
-        <is>
-          <t>Trasferimento</t>
-        </is>
-      </c>
+      <c r="A38" s="18" t="n"/>
+      <c r="B38" s="19" t="n"/>
+      <c r="C38" s="23" t="n"/>
+      <c r="D38" s="19" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="15" t="n">
-        <v>46284</v>
-      </c>
-      <c r="B39" s="17" t="inlineStr">
-        <is>
-          <t>EdenRed — Tigros (3 buoni pasto)</t>
-        </is>
-      </c>
-      <c r="C39" s="26" t="n">
-        <v>-27</v>
-      </c>
-      <c r="D39" s="17" t="inlineStr">
-        <is>
-          <t>Cibo</t>
-        </is>
-      </c>
+      <c r="A39" s="18" t="n"/>
+      <c r="B39" s="19" t="n"/>
+      <c r="C39" s="23" t="n"/>
+      <c r="D39" s="19" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="15" t="n">
-        <v>46284</v>
-      </c>
-      <c r="B40" s="17" t="inlineStr">
-        <is>
-          <t>EdenRed — 2 movimenti non dettagliati (4 buoni pasto)</t>
-        </is>
-      </c>
-      <c r="C40" s="26" t="n">
-        <v>-36</v>
-      </c>
-      <c r="D40" s="17" t="inlineStr">
-        <is>
-          <t>Cibo</t>
-        </is>
-      </c>
+      <c r="A40" s="18" t="n"/>
+      <c r="B40" s="19" t="n"/>
+      <c r="C40" s="23" t="n"/>
+      <c r="D40" s="19" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="18" t="n"/>
       <c r="B41" s="19" t="n"/>
-      <c r="C41" s="27" t="n"/>
+      <c r="C41" s="23" t="n"/>
       <c r="D41" s="19" t="n"/>
     </row>
-    <row r="42" ht="50" customHeight="1">
-      <c r="A42" s="28" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="B42" s="9" t="inlineStr">
-        <is>
-          <t>«Da verificare» = esercizio non riconosciuto dalla descrizione: chiedi conferma prima di riclassificarlo. «Trasferimento» = spostamenti fra tuoi conti/chiusura BCC Caravaggio: non sono spesa reale, per questo restano fuori dal totale. Le 4 ricariche buoni pasto del 19/09 non erano nello screenshot: importo dedotto da 21 caricati − 9 rimasti − gli 8 già visti = 4.</t>
-        </is>
-      </c>
+    <row r="42">
+      <c r="A42" s="18" t="n"/>
+      <c r="B42" s="19" t="n"/>
+      <c r="C42" s="23" t="n"/>
+      <c r="D42" s="19" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="18" t="n"/>
       <c r="B43" s="19" t="n"/>
-      <c r="C43" s="27" t="n"/>
+      <c r="C43" s="23" t="n"/>
       <c r="D43" s="19" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="18" t="n"/>
       <c r="B44" s="19" t="n"/>
-      <c r="C44" s="27" t="n"/>
+      <c r="C44" s="23" t="n"/>
       <c r="D44" s="19" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="18" t="n"/>
       <c r="B45" s="19" t="n"/>
-      <c r="C45" s="27" t="n"/>
+      <c r="C45" s="23" t="n"/>
       <c r="D45" s="19" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="18" t="n"/>
       <c r="B46" s="19" t="n"/>
-      <c r="C46" s="27" t="n"/>
+      <c r="C46" s="23" t="n"/>
       <c r="D46" s="19" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="18" t="n"/>
       <c r="B47" s="19" t="n"/>
-      <c r="C47" s="27" t="n"/>
+      <c r="C47" s="23" t="n"/>
       <c r="D47" s="19" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="18" t="n"/>
       <c r="B48" s="19" t="n"/>
-      <c r="C48" s="27" t="n"/>
+      <c r="C48" s="23" t="n"/>
       <c r="D48" s="19" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="18" t="n"/>
       <c r="B49" s="19" t="n"/>
-      <c r="C49" s="27" t="n"/>
+      <c r="C49" s="23" t="n"/>
       <c r="D49" s="19" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="18" t="n"/>
       <c r="B50" s="19" t="n"/>
-      <c r="C50" s="27" t="n"/>
+      <c r="C50" s="23" t="n"/>
       <c r="D50" s="19" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="18" t="n"/>
       <c r="B51" s="19" t="n"/>
-      <c r="C51" s="27" t="n"/>
+      <c r="C51" s="23" t="n"/>
       <c r="D51" s="19" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="18" t="n"/>
       <c r="B52" s="19" t="n"/>
-      <c r="C52" s="27" t="n"/>
+      <c r="C52" s="23" t="n"/>
       <c r="D52" s="19" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="18" t="n"/>
       <c r="B53" s="19" t="n"/>
-      <c r="C53" s="27" t="n"/>
+      <c r="C53" s="23" t="n"/>
       <c r="D53" s="19" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="18" t="n"/>
       <c r="B54" s="19" t="n"/>
-      <c r="C54" s="27" t="n"/>
+      <c r="C54" s="23" t="n"/>
       <c r="D54" s="19" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="18" t="n"/>
       <c r="B55" s="19" t="n"/>
-      <c r="C55" s="27" t="n"/>
+      <c r="C55" s="23" t="n"/>
       <c r="D55" s="19" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="18" t="n"/>
       <c r="B56" s="19" t="n"/>
-      <c r="C56" s="27" t="n"/>
+      <c r="C56" s="23" t="n"/>
       <c r="D56" s="19" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="18" t="n"/>
       <c r="B57" s="19" t="n"/>
-      <c r="C57" s="27" t="n"/>
+      <c r="C57" s="23" t="n"/>
       <c r="D57" s="19" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="18" t="n"/>
       <c r="B58" s="19" t="n"/>
-      <c r="C58" s="27" t="n"/>
+      <c r="C58" s="23" t="n"/>
       <c r="D58" s="19" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="18" t="n"/>
       <c r="B59" s="19" t="n"/>
-      <c r="C59" s="27" t="n"/>
+      <c r="C59" s="23" t="n"/>
       <c r="D59" s="19" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="18" t="n"/>
       <c r="B60" s="19" t="n"/>
-      <c r="C60" s="27" t="n"/>
+      <c r="C60" s="23" t="n"/>
       <c r="D60" s="19" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="18" t="n"/>
       <c r="B61" s="19" t="n"/>
-      <c r="C61" s="27" t="n"/>
+      <c r="C61" s="23" t="n"/>
       <c r="D61" s="19" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="18" t="n"/>
       <c r="B62" s="19" t="n"/>
-      <c r="C62" s="27" t="n"/>
+      <c r="C62" s="23" t="n"/>
       <c r="D62" s="19" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="18" t="n"/>
       <c r="B63" s="19" t="n"/>
-      <c r="C63" s="27" t="n"/>
+      <c r="C63" s="23" t="n"/>
       <c r="D63" s="19" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="18" t="n"/>
       <c r="B64" s="19" t="n"/>
-      <c r="C64" s="27" t="n"/>
+      <c r="C64" s="23" t="n"/>
       <c r="D64" s="19" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="18" t="n"/>
       <c r="B65" s="19" t="n"/>
-      <c r="C65" s="27" t="n"/>
+      <c r="C65" s="23" t="n"/>
       <c r="D65" s="19" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="18" t="n"/>
       <c r="B66" s="19" t="n"/>
-      <c r="C66" s="27" t="n"/>
+      <c r="C66" s="23" t="n"/>
       <c r="D66" s="19" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="18" t="n"/>
       <c r="B67" s="19" t="n"/>
-      <c r="C67" s="27" t="n"/>
+      <c r="C67" s="23" t="n"/>
       <c r="D67" s="19" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="18" t="n"/>
       <c r="B68" s="19" t="n"/>
-      <c r="C68" s="27" t="n"/>
+      <c r="C68" s="23" t="n"/>
       <c r="D68" s="19" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="18" t="n"/>
       <c r="B69" s="19" t="n"/>
-      <c r="C69" s="27" t="n"/>
+      <c r="C69" s="23" t="n"/>
       <c r="D69" s="19" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="18" t="n"/>
       <c r="B70" s="19" t="n"/>
-      <c r="C70" s="27" t="n"/>
+      <c r="C70" s="23" t="n"/>
       <c r="D70" s="19" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="18" t="n"/>
       <c r="B71" s="19" t="n"/>
-      <c r="C71" s="27" t="n"/>
+      <c r="C71" s="23" t="n"/>
       <c r="D71" s="19" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="18" t="n"/>
       <c r="B72" s="19" t="n"/>
-      <c r="C72" s="27" t="n"/>
+      <c r="C72" s="23" t="n"/>
       <c r="D72" s="19" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="18" t="n"/>
       <c r="B73" s="19" t="n"/>
-      <c r="C73" s="27" t="n"/>
+      <c r="C73" s="23" t="n"/>
       <c r="D73" s="19" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="18" t="n"/>
       <c r="B74" s="19" t="n"/>
-      <c r="C74" s="27" t="n"/>
+      <c r="C74" s="23" t="n"/>
       <c r="D74" s="19" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="18" t="n"/>
       <c r="B75" s="19" t="n"/>
-      <c r="C75" s="27" t="n"/>
+      <c r="C75" s="23" t="n"/>
       <c r="D75" s="19" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="18" t="n"/>
       <c r="B76" s="19" t="n"/>
-      <c r="C76" s="27" t="n"/>
+      <c r="C76" s="23" t="n"/>
       <c r="D76" s="19" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="18" t="n"/>
       <c r="B77" s="19" t="n"/>
-      <c r="C77" s="27" t="n"/>
+      <c r="C77" s="23" t="n"/>
       <c r="D77" s="19" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="18" t="n"/>
       <c r="B78" s="19" t="n"/>
-      <c r="C78" s="27" t="n"/>
+      <c r="C78" s="23" t="n"/>
       <c r="D78" s="19" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="18" t="n"/>
       <c r="B79" s="19" t="n"/>
-      <c r="C79" s="27" t="n"/>
+      <c r="C79" s="23" t="n"/>
       <c r="D79" s="19" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="18" t="n"/>
       <c r="B80" s="19" t="n"/>
-      <c r="C80" s="27" t="n"/>
+      <c r="C80" s="23" t="n"/>
       <c r="D80" s="19" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="18" t="n"/>
       <c r="B81" s="19" t="n"/>
-      <c r="C81" s="27" t="n"/>
+      <c r="C81" s="23" t="n"/>
       <c r="D81" s="19" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="18" t="n"/>
       <c r="B82" s="19" t="n"/>
-      <c r="C82" s="27" t="n"/>
+      <c r="C82" s="23" t="n"/>
       <c r="D82" s="19" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="18" t="n"/>
       <c r="B83" s="19" t="n"/>
-      <c r="C83" s="27" t="n"/>
+      <c r="C83" s="23" t="n"/>
       <c r="D83" s="19" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="18" t="n"/>
       <c r="B84" s="19" t="n"/>
-      <c r="C84" s="27" t="n"/>
+      <c r="C84" s="23" t="n"/>
       <c r="D84" s="19" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="18" t="n"/>
       <c r="B85" s="19" t="n"/>
-      <c r="C85" s="27" t="n"/>
+      <c r="C85" s="23" t="n"/>
       <c r="D85" s="19" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="18" t="n"/>
       <c r="B86" s="19" t="n"/>
-      <c r="C86" s="27" t="n"/>
+      <c r="C86" s="23" t="n"/>
       <c r="D86" s="19" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="18" t="n"/>
       <c r="B87" s="19" t="n"/>
-      <c r="C87" s="27" t="n"/>
+      <c r="C87" s="23" t="n"/>
       <c r="D87" s="19" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="18" t="n"/>
       <c r="B88" s="19" t="n"/>
-      <c r="C88" s="27" t="n"/>
+      <c r="C88" s="23" t="n"/>
       <c r="D88" s="19" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="18" t="n"/>
       <c r="B89" s="19" t="n"/>
-      <c r="C89" s="27" t="n"/>
+      <c r="C89" s="23" t="n"/>
       <c r="D89" s="19" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="18" t="n"/>
       <c r="B90" s="19" t="n"/>
-      <c r="C90" s="27" t="n"/>
+      <c r="C90" s="23" t="n"/>
       <c r="D90" s="19" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="18" t="n"/>
       <c r="B91" s="19" t="n"/>
-      <c r="C91" s="27" t="n"/>
+      <c r="C91" s="23" t="n"/>
       <c r="D91" s="19" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="18" t="n"/>
       <c r="B92" s="19" t="n"/>
-      <c r="C92" s="27" t="n"/>
+      <c r="C92" s="23" t="n"/>
       <c r="D92" s="19" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="18" t="n"/>
       <c r="B93" s="19" t="n"/>
-      <c r="C93" s="27" t="n"/>
+      <c r="C93" s="23" t="n"/>
       <c r="D93" s="19" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="18" t="n"/>
       <c r="B94" s="19" t="n"/>
-      <c r="C94" s="27" t="n"/>
+      <c r="C94" s="23" t="n"/>
       <c r="D94" s="19" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="18" t="n"/>
       <c r="B95" s="19" t="n"/>
-      <c r="C95" s="27" t="n"/>
+      <c r="C95" s="23" t="n"/>
       <c r="D95" s="19" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="18" t="n"/>
       <c r="B96" s="19" t="n"/>
-      <c r="C96" s="27" t="n"/>
+      <c r="C96" s="23" t="n"/>
       <c r="D96" s="19" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="18" t="n"/>
       <c r="B97" s="19" t="n"/>
-      <c r="C97" s="27" t="n"/>
+      <c r="C97" s="23" t="n"/>
       <c r="D97" s="19" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="18" t="n"/>
       <c r="B98" s="19" t="n"/>
-      <c r="C98" s="27" t="n"/>
+      <c r="C98" s="23" t="n"/>
       <c r="D98" s="19" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="18" t="n"/>
       <c r="B99" s="19" t="n"/>
-      <c r="C99" s="27" t="n"/>
+      <c r="C99" s="23" t="n"/>
       <c r="D99" s="19" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="18" t="n"/>
       <c r="B100" s="19" t="n"/>
-      <c r="C100" s="27" t="n"/>
+      <c r="C100" s="23" t="n"/>
       <c r="D100" s="19" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="18" t="n"/>
       <c r="B101" s="19" t="n"/>
-      <c r="C101" s="27" t="n"/>
+      <c r="C101" s="23" t="n"/>
       <c r="D101" s="19" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="18" t="n"/>
       <c r="B102" s="19" t="n"/>
-      <c r="C102" s="27" t="n"/>
+      <c r="C102" s="23" t="n"/>
       <c r="D102" s="19" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="18" t="n"/>
       <c r="B103" s="19" t="n"/>
-      <c r="C103" s="27" t="n"/>
+      <c r="C103" s="23" t="n"/>
       <c r="D103" s="19" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="18" t="n"/>
       <c r="B104" s="19" t="n"/>
-      <c r="C104" s="27" t="n"/>
+      <c r="C104" s="23" t="n"/>
       <c r="D104" s="19" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="18" t="n"/>
       <c r="B105" s="19" t="n"/>
-      <c r="C105" s="27" t="n"/>
+      <c r="C105" s="23" t="n"/>
       <c r="D105" s="19" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="18" t="n"/>
       <c r="B106" s="19" t="n"/>
-      <c r="C106" s="27" t="n"/>
+      <c r="C106" s="23" t="n"/>
       <c r="D106" s="19" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="18" t="n"/>
       <c r="B107" s="19" t="n"/>
-      <c r="C107" s="27" t="n"/>
+      <c r="C107" s="23" t="n"/>
       <c r="D107" s="19" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="18" t="n"/>
       <c r="B108" s="19" t="n"/>
-      <c r="C108" s="27" t="n"/>
+      <c r="C108" s="23" t="n"/>
       <c r="D108" s="19" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="18" t="n"/>
       <c r="B109" s="19" t="n"/>
-      <c r="C109" s="27" t="n"/>
+      <c r="C109" s="23" t="n"/>
       <c r="D109" s="19" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="18" t="n"/>
       <c r="B110" s="19" t="n"/>
-      <c r="C110" s="27" t="n"/>
+      <c r="C110" s="23" t="n"/>
       <c r="D110" s="19" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="18" t="n"/>
       <c r="B111" s="19" t="n"/>
-      <c r="C111" s="27" t="n"/>
+      <c r="C111" s="23" t="n"/>
       <c r="D111" s="19" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="18" t="n"/>
       <c r="B112" s="19" t="n"/>
-      <c r="C112" s="27" t="n"/>
+      <c r="C112" s="23" t="n"/>
       <c r="D112" s="19" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="18" t="n"/>
       <c r="B113" s="19" t="n"/>
-      <c r="C113" s="27" t="n"/>
+      <c r="C113" s="23" t="n"/>
       <c r="D113" s="19" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="18" t="n"/>
       <c r="B114" s="19" t="n"/>
-      <c r="C114" s="27" t="n"/>
+      <c r="C114" s="23" t="n"/>
       <c r="D114" s="19" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="18" t="n"/>
       <c r="B115" s="19" t="n"/>
-      <c r="C115" s="27" t="n"/>
+      <c r="C115" s="23" t="n"/>
       <c r="D115" s="19" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="18" t="n"/>
       <c r="B116" s="19" t="n"/>
-      <c r="C116" s="27" t="n"/>
+      <c r="C116" s="23" t="n"/>
       <c r="D116" s="19" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="18" t="n"/>
       <c r="B117" s="19" t="n"/>
-      <c r="C117" s="27" t="n"/>
+      <c r="C117" s="23" t="n"/>
       <c r="D117" s="19" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="18" t="n"/>
       <c r="B118" s="19" t="n"/>
-      <c r="C118" s="27" t="n"/>
+      <c r="C118" s="23" t="n"/>
       <c r="D118" s="19" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="18" t="n"/>
       <c r="B119" s="19" t="n"/>
-      <c r="C119" s="27" t="n"/>
+      <c r="C119" s="23" t="n"/>
       <c r="D119" s="19" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="18" t="n"/>
       <c r="B120" s="19" t="n"/>
-      <c r="C120" s="27" t="n"/>
+      <c r="C120" s="23" t="n"/>
       <c r="D120" s="19" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="18" t="n"/>
       <c r="B121" s="19" t="n"/>
-      <c r="C121" s="27" t="n"/>
+      <c r="C121" s="23" t="n"/>
       <c r="D121" s="19" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="18" t="n"/>
       <c r="B122" s="19" t="n"/>
-      <c r="C122" s="27" t="n"/>
+      <c r="C122" s="23" t="n"/>
       <c r="D122" s="19" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="18" t="n"/>
       <c r="B123" s="19" t="n"/>
-      <c r="C123" s="27" t="n"/>
+      <c r="C123" s="23" t="n"/>
       <c r="D123" s="19" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="18" t="n"/>
       <c r="B124" s="19" t="n"/>
-      <c r="C124" s="27" t="n"/>
+      <c r="C124" s="23" t="n"/>
       <c r="D124" s="19" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="18" t="n"/>
       <c r="B125" s="19" t="n"/>
-      <c r="C125" s="27" t="n"/>
+      <c r="C125" s="23" t="n"/>
       <c r="D125" s="19" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="18" t="n"/>
       <c r="B126" s="19" t="n"/>
-      <c r="C126" s="27" t="n"/>
+      <c r="C126" s="23" t="n"/>
       <c r="D126" s="19" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="18" t="n"/>
       <c r="B127" s="19" t="n"/>
-      <c r="C127" s="27" t="n"/>
+      <c r="C127" s="23" t="n"/>
       <c r="D127" s="19" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="18" t="n"/>
       <c r="B128" s="19" t="n"/>
-      <c r="C128" s="27" t="n"/>
+      <c r="C128" s="23" t="n"/>
       <c r="D128" s="19" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="18" t="n"/>
       <c r="B129" s="19" t="n"/>
-      <c r="C129" s="27" t="n"/>
+      <c r="C129" s="23" t="n"/>
       <c r="D129" s="19" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="18" t="n"/>
       <c r="B130" s="19" t="n"/>
-      <c r="C130" s="27" t="n"/>
+      <c r="C130" s="23" t="n"/>
       <c r="D130" s="19" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="18" t="n"/>
       <c r="B131" s="19" t="n"/>
-      <c r="C131" s="27" t="n"/>
+      <c r="C131" s="23" t="n"/>
       <c r="D131" s="19" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="18" t="n"/>
       <c r="B132" s="19" t="n"/>
-      <c r="C132" s="27" t="n"/>
+      <c r="C132" s="23" t="n"/>
       <c r="D132" s="19" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="18" t="n"/>
       <c r="B133" s="19" t="n"/>
-      <c r="C133" s="27" t="n"/>
+      <c r="C133" s="23" t="n"/>
       <c r="D133" s="19" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="18" t="n"/>
       <c r="B134" s="19" t="n"/>
-      <c r="C134" s="27" t="n"/>
+      <c r="C134" s="23" t="n"/>
       <c r="D134" s="19" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="18" t="n"/>
       <c r="B135" s="19" t="n"/>
-      <c r="C135" s="27" t="n"/>
+      <c r="C135" s="23" t="n"/>
       <c r="D135" s="19" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="18" t="n"/>
       <c r="B136" s="19" t="n"/>
-      <c r="C136" s="27" t="n"/>
+      <c r="C136" s="23" t="n"/>
       <c r="D136" s="19" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="18" t="n"/>
       <c r="B137" s="19" t="n"/>
-      <c r="C137" s="27" t="n"/>
+      <c r="C137" s="23" t="n"/>
       <c r="D137" s="19" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="18" t="n"/>
       <c r="B138" s="19" t="n"/>
-      <c r="C138" s="27" t="n"/>
+      <c r="C138" s="23" t="n"/>
       <c r="D138" s="19" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="18" t="n"/>
       <c r="B139" s="19" t="n"/>
-      <c r="C139" s="27" t="n"/>
+      <c r="C139" s="23" t="n"/>
       <c r="D139" s="19" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="18" t="n"/>
       <c r="B140" s="19" t="n"/>
-      <c r="C140" s="27" t="n"/>
+      <c r="C140" s="23" t="n"/>
       <c r="D140" s="19" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="18" t="n"/>
       <c r="B141" s="19" t="n"/>
-      <c r="C141" s="27" t="n"/>
+      <c r="C141" s="23" t="n"/>
       <c r="D141" s="19" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="18" t="n"/>
       <c r="B142" s="19" t="n"/>
-      <c r="C142" s="27" t="n"/>
+      <c r="C142" s="23" t="n"/>
       <c r="D142" s="19" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="18" t="n"/>
       <c r="B143" s="19" t="n"/>
-      <c r="C143" s="27" t="n"/>
+      <c r="C143" s="23" t="n"/>
       <c r="D143" s="19" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="18" t="n"/>
       <c r="B144" s="19" t="n"/>
-      <c r="C144" s="27" t="n"/>
+      <c r="C144" s="23" t="n"/>
       <c r="D144" s="19" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="18" t="n"/>
       <c r="B145" s="19" t="n"/>
-      <c r="C145" s="27" t="n"/>
+      <c r="C145" s="23" t="n"/>
       <c r="D145" s="19" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="18" t="n"/>
       <c r="B146" s="19" t="n"/>
-      <c r="C146" s="27" t="n"/>
+      <c r="C146" s="23" t="n"/>
       <c r="D146" s="19" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="18" t="n"/>
       <c r="B147" s="19" t="n"/>
-      <c r="C147" s="27" t="n"/>
+      <c r="C147" s="23" t="n"/>
       <c r="D147" s="19" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="18" t="n"/>
       <c r="B148" s="19" t="n"/>
-      <c r="C148" s="27" t="n"/>
+      <c r="C148" s="23" t="n"/>
       <c r="D148" s="19" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="18" t="n"/>
       <c r="B149" s="19" t="n"/>
-      <c r="C149" s="27" t="n"/>
+      <c r="C149" s="23" t="n"/>
       <c r="D149" s="19" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="18" t="n"/>
       <c r="B150" s="19" t="n"/>
-      <c r="C150" s="27" t="n"/>
+      <c r="C150" s="23" t="n"/>
       <c r="D150" s="19" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="18" t="n"/>
       <c r="B151" s="19" t="n"/>
-      <c r="C151" s="27" t="n"/>
+      <c r="C151" s="23" t="n"/>
       <c r="D151" s="19" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="18" t="n"/>
       <c r="B152" s="19" t="n"/>
-      <c r="C152" s="27" t="n"/>
+      <c r="C152" s="23" t="n"/>
       <c r="D152" s="19" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="18" t="n"/>
       <c r="B153" s="19" t="n"/>
-      <c r="C153" s="27" t="n"/>
+      <c r="C153" s="23" t="n"/>
       <c r="D153" s="19" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="18" t="n"/>
       <c r="B154" s="19" t="n"/>
-      <c r="C154" s="27" t="n"/>
+      <c r="C154" s="23" t="n"/>
       <c r="D154" s="19" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="18" t="n"/>
       <c r="B155" s="19" t="n"/>
-      <c r="C155" s="27" t="n"/>
+      <c r="C155" s="23" t="n"/>
       <c r="D155" s="19" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="18" t="n"/>
       <c r="B156" s="19" t="n"/>
-      <c r="C156" s="27" t="n"/>
+      <c r="C156" s="23" t="n"/>
       <c r="D156" s="19" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="18" t="n"/>
       <c r="B157" s="19" t="n"/>
-      <c r="C157" s="27" t="n"/>
+      <c r="C157" s="23" t="n"/>
       <c r="D157" s="19" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="18" t="n"/>
       <c r="B158" s="19" t="n"/>
-      <c r="C158" s="27" t="n"/>
+      <c r="C158" s="23" t="n"/>
       <c r="D158" s="19" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="18" t="n"/>
       <c r="B159" s="19" t="n"/>
-      <c r="C159" s="27" t="n"/>
+      <c r="C159" s="23" t="n"/>
       <c r="D159" s="19" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="18" t="n"/>
       <c r="B160" s="19" t="n"/>
-      <c r="C160" s="27" t="n"/>
+      <c r="C160" s="23" t="n"/>
       <c r="D160" s="19" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="18" t="n"/>
       <c r="B161" s="19" t="n"/>
-      <c r="C161" s="27" t="n"/>
+      <c r="C161" s="23" t="n"/>
       <c r="D161" s="19" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="18" t="n"/>
       <c r="B162" s="19" t="n"/>
-      <c r="C162" s="27" t="n"/>
+      <c r="C162" s="23" t="n"/>
       <c r="D162" s="19" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="18" t="n"/>
       <c r="B163" s="19" t="n"/>
-      <c r="C163" s="27" t="n"/>
+      <c r="C163" s="23" t="n"/>
       <c r="D163" s="19" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="18" t="n"/>
       <c r="B164" s="19" t="n"/>
-      <c r="C164" s="27" t="n"/>
+      <c r="C164" s="23" t="n"/>
       <c r="D164" s="19" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="18" t="n"/>
       <c r="B165" s="19" t="n"/>
-      <c r="C165" s="27" t="n"/>
+      <c r="C165" s="23" t="n"/>
       <c r="D165" s="19" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="18" t="n"/>
       <c r="B166" s="19" t="n"/>
-      <c r="C166" s="27" t="n"/>
+      <c r="C166" s="23" t="n"/>
       <c r="D166" s="19" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="18" t="n"/>
       <c r="B167" s="19" t="n"/>
-      <c r="C167" s="27" t="n"/>
+      <c r="C167" s="23" t="n"/>
       <c r="D167" s="19" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="18" t="n"/>
       <c r="B168" s="19" t="n"/>
-      <c r="C168" s="27" t="n"/>
+      <c r="C168" s="23" t="n"/>
       <c r="D168" s="19" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="18" t="n"/>
       <c r="B169" s="19" t="n"/>
-      <c r="C169" s="27" t="n"/>
+      <c r="C169" s="23" t="n"/>
       <c r="D169" s="19" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="18" t="n"/>
       <c r="B170" s="19" t="n"/>
-      <c r="C170" s="27" t="n"/>
+      <c r="C170" s="23" t="n"/>
       <c r="D170" s="19" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="18" t="n"/>
       <c r="B171" s="19" t="n"/>
-      <c r="C171" s="27" t="n"/>
+      <c r="C171" s="23" t="n"/>
       <c r="D171" s="19" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="18" t="n"/>
       <c r="B172" s="19" t="n"/>
-      <c r="C172" s="27" t="n"/>
+      <c r="C172" s="23" t="n"/>
       <c r="D172" s="19" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="18" t="n"/>
       <c r="B173" s="19" t="n"/>
-      <c r="C173" s="27" t="n"/>
+      <c r="C173" s="23" t="n"/>
       <c r="D173" s="19" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="18" t="n"/>
       <c r="B174" s="19" t="n"/>
-      <c r="C174" s="27" t="n"/>
+      <c r="C174" s="23" t="n"/>
       <c r="D174" s="19" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="18" t="n"/>
       <c r="B175" s="19" t="n"/>
-      <c r="C175" s="27" t="n"/>
+      <c r="C175" s="23" t="n"/>
       <c r="D175" s="19" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="18" t="n"/>
       <c r="B176" s="19" t="n"/>
-      <c r="C176" s="27" t="n"/>
+      <c r="C176" s="23" t="n"/>
       <c r="D176" s="19" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="18" t="n"/>
       <c r="B177" s="19" t="n"/>
-      <c r="C177" s="27" t="n"/>
+      <c r="C177" s="23" t="n"/>
       <c r="D177" s="19" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="18" t="n"/>
       <c r="B178" s="19" t="n"/>
-      <c r="C178" s="27" t="n"/>
+      <c r="C178" s="23" t="n"/>
       <c r="D178" s="19" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="18" t="n"/>
       <c r="B179" s="19" t="n"/>
-      <c r="C179" s="27" t="n"/>
+      <c r="C179" s="23" t="n"/>
       <c r="D179" s="19" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="18" t="n"/>
       <c r="B180" s="19" t="n"/>
-      <c r="C180" s="27" t="n"/>
+      <c r="C180" s="23" t="n"/>
       <c r="D180" s="19" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="18" t="n"/>
       <c r="B181" s="19" t="n"/>
-      <c r="C181" s="27" t="n"/>
+      <c r="C181" s="23" t="n"/>
       <c r="D181" s="19" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="18" t="n"/>
       <c r="B182" s="19" t="n"/>
-      <c r="C182" s="27" t="n"/>
+      <c r="C182" s="23" t="n"/>
       <c r="D182" s="19" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="18" t="n"/>
       <c r="B183" s="19" t="n"/>
-      <c r="C183" s="27" t="n"/>
+      <c r="C183" s="23" t="n"/>
       <c r="D183" s="19" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="18" t="n"/>
       <c r="B184" s="19" t="n"/>
-      <c r="C184" s="27" t="n"/>
+      <c r="C184" s="23" t="n"/>
       <c r="D184" s="19" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="18" t="n"/>
       <c r="B185" s="19" t="n"/>
-      <c r="C185" s="27" t="n"/>
+      <c r="C185" s="23" t="n"/>
       <c r="D185" s="19" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="18" t="n"/>
       <c r="B186" s="19" t="n"/>
-      <c r="C186" s="27" t="n"/>
+      <c r="C186" s="23" t="n"/>
       <c r="D186" s="19" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="18" t="n"/>
       <c r="B187" s="19" t="n"/>
-      <c r="C187" s="27" t="n"/>
+      <c r="C187" s="23" t="n"/>
       <c r="D187" s="19" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="18" t="n"/>
       <c r="B188" s="19" t="n"/>
-      <c r="C188" s="27" t="n"/>
+      <c r="C188" s="23" t="n"/>
       <c r="D188" s="19" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="18" t="n"/>
       <c r="B189" s="19" t="n"/>
-      <c r="C189" s="27" t="n"/>
+      <c r="C189" s="23" t="n"/>
       <c r="D189" s="19" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="18" t="n"/>
       <c r="B190" s="19" t="n"/>
-      <c r="C190" s="27" t="n"/>
+      <c r="C190" s="23" t="n"/>
       <c r="D190" s="19" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="18" t="n"/>
       <c r="B191" s="19" t="n"/>
-      <c r="C191" s="27" t="n"/>
+      <c r="C191" s="23" t="n"/>
       <c r="D191" s="19" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="18" t="n"/>
       <c r="B192" s="19" t="n"/>
-      <c r="C192" s="27" t="n"/>
+      <c r="C192" s="23" t="n"/>
       <c r="D192" s="19" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="18" t="n"/>
       <c r="B193" s="19" t="n"/>
-      <c r="C193" s="27" t="n"/>
+      <c r="C193" s="23" t="n"/>
       <c r="D193" s="19" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="18" t="n"/>
       <c r="B194" s="19" t="n"/>
-      <c r="C194" s="27" t="n"/>
+      <c r="C194" s="23" t="n"/>
       <c r="D194" s="19" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="18" t="n"/>
       <c r="B195" s="19" t="n"/>
-      <c r="C195" s="27" t="n"/>
+      <c r="C195" s="23" t="n"/>
       <c r="D195" s="19" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="18" t="n"/>
       <c r="B196" s="19" t="n"/>
-      <c r="C196" s="27" t="n"/>
+      <c r="C196" s="23" t="n"/>
       <c r="D196" s="19" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="18" t="n"/>
       <c r="B197" s="19" t="n"/>
-      <c r="C197" s="27" t="n"/>
+      <c r="C197" s="23" t="n"/>
       <c r="D197" s="19" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="18" t="n"/>
       <c r="B198" s="19" t="n"/>
-      <c r="C198" s="27" t="n"/>
+      <c r="C198" s="23" t="n"/>
       <c r="D198" s="19" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="18" t="n"/>
       <c r="B199" s="19" t="n"/>
-      <c r="C199" s="27" t="n"/>
+      <c r="C199" s="23" t="n"/>
       <c r="D199" s="19" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="18" t="n"/>
       <c r="B200" s="19" t="n"/>
-      <c r="C200" s="27" t="n"/>
+      <c r="C200" s="23" t="n"/>
       <c r="D200" s="19" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="18" t="n"/>
       <c r="B201" s="19" t="n"/>
-      <c r="C201" s="27" t="n"/>
+      <c r="C201" s="23" t="n"/>
       <c r="D201" s="19" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="18" t="n"/>
       <c r="B202" s="19" t="n"/>
-      <c r="C202" s="27" t="n"/>
+      <c r="C202" s="23" t="n"/>
       <c r="D202" s="19" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="18" t="n"/>
       <c r="B203" s="19" t="n"/>
-      <c r="C203" s="27" t="n"/>
+      <c r="C203" s="23" t="n"/>
       <c r="D203" s="19" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="18" t="n"/>
       <c r="B204" s="19" t="n"/>
-      <c r="C204" s="27" t="n"/>
+      <c r="C204" s="23" t="n"/>
       <c r="D204" s="19" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="18" t="n"/>
       <c r="B205" s="19" t="n"/>
-      <c r="C205" s="27" t="n"/>
+      <c r="C205" s="23" t="n"/>
       <c r="D205" s="19" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="18" t="n"/>
       <c r="B206" s="19" t="n"/>
-      <c r="C206" s="27" t="n"/>
+      <c r="C206" s="23" t="n"/>
       <c r="D206" s="19" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="18" t="n"/>
       <c r="B207" s="19" t="n"/>
-      <c r="C207" s="27" t="n"/>
+      <c r="C207" s="23" t="n"/>
       <c r="D207" s="19" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="18" t="n"/>
       <c r="B208" s="19" t="n"/>
-      <c r="C208" s="27" t="n"/>
+      <c r="C208" s="23" t="n"/>
       <c r="D208" s="19" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="18" t="n"/>
       <c r="B209" s="19" t="n"/>
-      <c r="C209" s="27" t="n"/>
+      <c r="C209" s="23" t="n"/>
       <c r="D209" s="19" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="18" t="n"/>
       <c r="B210" s="19" t="n"/>
-      <c r="C210" s="27" t="n"/>
+      <c r="C210" s="23" t="n"/>
       <c r="D210" s="19" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="18" t="n"/>
       <c r="B211" s="19" t="n"/>
-      <c r="C211" s="27" t="n"/>
+      <c r="C211" s="23" t="n"/>
       <c r="D211" s="19" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="18" t="n"/>
       <c r="B212" s="19" t="n"/>
-      <c r="C212" s="27" t="n"/>
+      <c r="C212" s="23" t="n"/>
       <c r="D212" s="19" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="18" t="n"/>
       <c r="B213" s="19" t="n"/>
-      <c r="C213" s="27" t="n"/>
+      <c r="C213" s="23" t="n"/>
       <c r="D213" s="19" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="18" t="n"/>
       <c r="B214" s="19" t="n"/>
-      <c r="C214" s="27" t="n"/>
+      <c r="C214" s="23" t="n"/>
       <c r="D214" s="19" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="18" t="n"/>
       <c r="B215" s="19" t="n"/>
-      <c r="C215" s="27" t="n"/>
+      <c r="C215" s="23" t="n"/>
       <c r="D215" s="19" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="18" t="n"/>
       <c r="B216" s="19" t="n"/>
-      <c r="C216" s="27" t="n"/>
+      <c r="C216" s="23" t="n"/>
       <c r="D216" s="19" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="18" t="n"/>
       <c r="B217" s="19" t="n"/>
-      <c r="C217" s="27" t="n"/>
+      <c r="C217" s="23" t="n"/>
       <c r="D217" s="19" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="18" t="n"/>
       <c r="B218" s="19" t="n"/>
-      <c r="C218" s="27" t="n"/>
+      <c r="C218" s="23" t="n"/>
       <c r="D218" s="19" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="18" t="n"/>
       <c r="B219" s="19" t="n"/>
-      <c r="C219" s="27" t="n"/>
+      <c r="C219" s="23" t="n"/>
       <c r="D219" s="19" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="18" t="n"/>
       <c r="B220" s="19" t="n"/>
-      <c r="C220" s="27" t="n"/>
+      <c r="C220" s="23" t="n"/>
       <c r="D220" s="19" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="18" t="n"/>
       <c r="B221" s="19" t="n"/>
-      <c r="C221" s="27" t="n"/>
+      <c r="C221" s="23" t="n"/>
       <c r="D221" s="19" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="18" t="n"/>
       <c r="B222" s="19" t="n"/>
-      <c r="C222" s="27" t="n"/>
+      <c r="C222" s="23" t="n"/>
       <c r="D222" s="19" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="18" t="n"/>
       <c r="B223" s="19" t="n"/>
-      <c r="C223" s="27" t="n"/>
+      <c r="C223" s="23" t="n"/>
       <c r="D223" s="19" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="18" t="n"/>
       <c r="B224" s="19" t="n"/>
-      <c r="C224" s="27" t="n"/>
+      <c r="C224" s="23" t="n"/>
       <c r="D224" s="19" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="18" t="n"/>
       <c r="B225" s="19" t="n"/>
-      <c r="C225" s="27" t="n"/>
+      <c r="C225" s="23" t="n"/>
       <c r="D225" s="19" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="18" t="n"/>
       <c r="B226" s="19" t="n"/>
-      <c r="C226" s="27" t="n"/>
+      <c r="C226" s="23" t="n"/>
       <c r="D226" s="19" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="18" t="n"/>
       <c r="B227" s="19" t="n"/>
-      <c r="C227" s="27" t="n"/>
+      <c r="C227" s="23" t="n"/>
       <c r="D227" s="19" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="18" t="n"/>
       <c r="B228" s="19" t="n"/>
-      <c r="C228" s="27" t="n"/>
+      <c r="C228" s="23" t="n"/>
       <c r="D228" s="19" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="18" t="n"/>
       <c r="B229" s="19" t="n"/>
-      <c r="C229" s="27" t="n"/>
+      <c r="C229" s="23" t="n"/>
       <c r="D229" s="19" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="18" t="n"/>
       <c r="B230" s="19" t="n"/>
-      <c r="C230" s="27" t="n"/>
+      <c r="C230" s="23" t="n"/>
       <c r="D230" s="19" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="18" t="n"/>
       <c r="B231" s="19" t="n"/>
-      <c r="C231" s="27" t="n"/>
+      <c r="C231" s="23" t="n"/>
       <c r="D231" s="19" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="18" t="n"/>
       <c r="B232" s="19" t="n"/>
-      <c r="C232" s="27" t="n"/>
+      <c r="C232" s="23" t="n"/>
       <c r="D232" s="19" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="18" t="n"/>
       <c r="B233" s="19" t="n"/>
-      <c r="C233" s="27" t="n"/>
+      <c r="C233" s="23" t="n"/>
       <c r="D233" s="19" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="18" t="n"/>
       <c r="B234" s="19" t="n"/>
-      <c r="C234" s="27" t="n"/>
+      <c r="C234" s="23" t="n"/>
       <c r="D234" s="19" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="18" t="n"/>
       <c r="B235" s="19" t="n"/>
-      <c r="C235" s="27" t="n"/>
+      <c r="C235" s="23" t="n"/>
       <c r="D235" s="19" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="18" t="n"/>
       <c r="B236" s="19" t="n"/>
-      <c r="C236" s="27" t="n"/>
+      <c r="C236" s="23" t="n"/>
       <c r="D236" s="19" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="18" t="n"/>
       <c r="B237" s="19" t="n"/>
-      <c r="C237" s="27" t="n"/>
+      <c r="C237" s="23" t="n"/>
       <c r="D237" s="19" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="18" t="n"/>
       <c r="B238" s="19" t="n"/>
-      <c r="C238" s="27" t="n"/>
+      <c r="C238" s="23" t="n"/>
       <c r="D238" s="19" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="18" t="n"/>
       <c r="B239" s="19" t="n"/>
-      <c r="C239" s="27" t="n"/>
+      <c r="C239" s="23" t="n"/>
       <c r="D239" s="19" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="18" t="n"/>
       <c r="B240" s="19" t="n"/>
-      <c r="C240" s="27" t="n"/>
+      <c r="C240" s="23" t="n"/>
       <c r="D240" s="19" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="18" t="n"/>
       <c r="B241" s="19" t="n"/>
-      <c r="C241" s="27" t="n"/>
+      <c r="C241" s="23" t="n"/>
       <c r="D241" s="19" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="18" t="n"/>
       <c r="B242" s="19" t="n"/>
-      <c r="C242" s="27" t="n"/>
+      <c r="C242" s="23" t="n"/>
       <c r="D242" s="19" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="18" t="n"/>
       <c r="B243" s="19" t="n"/>
-      <c r="C243" s="27" t="n"/>
+      <c r="C243" s="23" t="n"/>
       <c r="D243" s="19" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="18" t="n"/>
       <c r="B244" s="19" t="n"/>
-      <c r="C244" s="27" t="n"/>
+      <c r="C244" s="23" t="n"/>
       <c r="D244" s="19" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="18" t="n"/>
       <c r="B245" s="19" t="n"/>
-      <c r="C245" s="27" t="n"/>
+      <c r="C245" s="23" t="n"/>
       <c r="D245" s="19" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="18" t="n"/>
       <c r="B246" s="19" t="n"/>
-      <c r="C246" s="27" t="n"/>
+      <c r="C246" s="23" t="n"/>
       <c r="D246" s="19" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="18" t="n"/>
       <c r="B247" s="19" t="n"/>
-      <c r="C247" s="27" t="n"/>
+      <c r="C247" s="23" t="n"/>
       <c r="D247" s="19" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="18" t="n"/>
       <c r="B248" s="19" t="n"/>
-      <c r="C248" s="27" t="n"/>
+      <c r="C248" s="23" t="n"/>
       <c r="D248" s="19" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="18" t="n"/>
       <c r="B249" s="19" t="n"/>
-      <c r="C249" s="27" t="n"/>
+      <c r="C249" s="23" t="n"/>
       <c r="D249" s="19" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="18" t="n"/>
       <c r="B250" s="19" t="n"/>
-      <c r="C250" s="27" t="n"/>
+      <c r="C250" s="23" t="n"/>
       <c r="D250" s="19" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="18" t="n"/>
       <c r="B251" s="19" t="n"/>
-      <c r="C251" s="27" t="n"/>
+      <c r="C251" s="23" t="n"/>
       <c r="D251" s="19" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="18" t="n"/>
       <c r="B252" s="19" t="n"/>
-      <c r="C252" s="27" t="n"/>
+      <c r="C252" s="23" t="n"/>
       <c r="D252" s="19" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="18" t="n"/>
       <c r="B253" s="19" t="n"/>
-      <c r="C253" s="27" t="n"/>
+      <c r="C253" s="23" t="n"/>
       <c r="D253" s="19" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="18" t="n"/>
       <c r="B254" s="19" t="n"/>
-      <c r="C254" s="27" t="n"/>
+      <c r="C254" s="23" t="n"/>
       <c r="D254" s="19" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="18" t="n"/>
       <c r="B255" s="19" t="n"/>
-      <c r="C255" s="27" t="n"/>
+      <c r="C255" s="23" t="n"/>
       <c r="D255" s="19" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="18" t="n"/>
       <c r="B256" s="19" t="n"/>
-      <c r="C256" s="27" t="n"/>
+      <c r="C256" s="23" t="n"/>
       <c r="D256" s="19" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="18" t="n"/>
       <c r="B257" s="19" t="n"/>
-      <c r="C257" s="27" t="n"/>
+      <c r="C257" s="23" t="n"/>
       <c r="D257" s="19" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="18" t="n"/>
       <c r="B258" s="19" t="n"/>
-      <c r="C258" s="27" t="n"/>
+      <c r="C258" s="23" t="n"/>
       <c r="D258" s="19" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="18" t="n"/>
       <c r="B259" s="19" t="n"/>
-      <c r="C259" s="27" t="n"/>
+      <c r="C259" s="23" t="n"/>
       <c r="D259" s="19" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="18" t="n"/>
       <c r="B260" s="19" t="n"/>
-      <c r="C260" s="27" t="n"/>
+      <c r="C260" s="23" t="n"/>
       <c r="D260" s="19" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="18" t="n"/>
       <c r="B261" s="19" t="n"/>
-      <c r="C261" s="27" t="n"/>
+      <c r="C261" s="23" t="n"/>
       <c r="D261" s="19" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="18" t="n"/>
       <c r="B262" s="19" t="n"/>
-      <c r="C262" s="27" t="n"/>
+      <c r="C262" s="23" t="n"/>
       <c r="D262" s="19" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="18" t="n"/>
       <c r="B263" s="19" t="n"/>
-      <c r="C263" s="27" t="n"/>
+      <c r="C263" s="23" t="n"/>
       <c r="D263" s="19" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="18" t="n"/>
       <c r="B264" s="19" t="n"/>
-      <c r="C264" s="27" t="n"/>
+      <c r="C264" s="23" t="n"/>
       <c r="D264" s="19" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="18" t="n"/>
       <c r="B265" s="19" t="n"/>
-      <c r="C265" s="27" t="n"/>
+      <c r="C265" s="23" t="n"/>
       <c r="D265" s="19" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="18" t="n"/>
       <c r="B266" s="19" t="n"/>
-      <c r="C266" s="27" t="n"/>
+      <c r="C266" s="23" t="n"/>
       <c r="D266" s="19" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="18" t="n"/>
       <c r="B267" s="19" t="n"/>
-      <c r="C267" s="27" t="n"/>
+      <c r="C267" s="23" t="n"/>
       <c r="D267" s="19" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="18" t="n"/>
       <c r="B268" s="19" t="n"/>
-      <c r="C268" s="27" t="n"/>
+      <c r="C268" s="23" t="n"/>
       <c r="D268" s="19" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="18" t="n"/>
       <c r="B269" s="19" t="n"/>
-      <c r="C269" s="27" t="n"/>
+      <c r="C269" s="23" t="n"/>
       <c r="D269" s="19" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="18" t="n"/>
       <c r="B270" s="19" t="n"/>
-      <c r="C270" s="27" t="n"/>
+      <c r="C270" s="23" t="n"/>
       <c r="D270" s="19" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="18" t="n"/>
       <c r="B271" s="19" t="n"/>
-      <c r="C271" s="27" t="n"/>
+      <c r="C271" s="23" t="n"/>
       <c r="D271" s="19" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="18" t="n"/>
       <c r="B272" s="19" t="n"/>
-      <c r="C272" s="27" t="n"/>
+      <c r="C272" s="23" t="n"/>
       <c r="D272" s="19" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="18" t="n"/>
       <c r="B273" s="19" t="n"/>
-      <c r="C273" s="27" t="n"/>
+      <c r="C273" s="23" t="n"/>
       <c r="D273" s="19" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="18" t="n"/>
       <c r="B274" s="19" t="n"/>
-      <c r="C274" s="27" t="n"/>
+      <c r="C274" s="23" t="n"/>
       <c r="D274" s="19" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="18" t="n"/>
       <c r="B275" s="19" t="n"/>
-      <c r="C275" s="27" t="n"/>
+      <c r="C275" s="23" t="n"/>
       <c r="D275" s="19" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="18" t="n"/>
       <c r="B276" s="19" t="n"/>
-      <c r="C276" s="27" t="n"/>
+      <c r="C276" s="23" t="n"/>
       <c r="D276" s="19" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="18" t="n"/>
       <c r="B277" s="19" t="n"/>
-      <c r="C277" s="27" t="n"/>
+      <c r="C277" s="23" t="n"/>
       <c r="D277" s="19" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="18" t="n"/>
       <c r="B278" s="19" t="n"/>
-      <c r="C278" s="27" t="n"/>
+      <c r="C278" s="23" t="n"/>
       <c r="D278" s="19" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="18" t="n"/>
       <c r="B279" s="19" t="n"/>
-      <c r="C279" s="27" t="n"/>
+      <c r="C279" s="23" t="n"/>
       <c r="D279" s="19" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="18" t="n"/>
       <c r="B280" s="19" t="n"/>
-      <c r="C280" s="27" t="n"/>
+      <c r="C280" s="23" t="n"/>
       <c r="D280" s="19" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="18" t="n"/>
       <c r="B281" s="19" t="n"/>
-      <c r="C281" s="27" t="n"/>
+      <c r="C281" s="23" t="n"/>
       <c r="D281" s="19" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="18" t="n"/>
       <c r="B282" s="19" t="n"/>
-      <c r="C282" s="27" t="n"/>
+      <c r="C282" s="23" t="n"/>
       <c r="D282" s="19" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="18" t="n"/>
       <c r="B283" s="19" t="n"/>
-      <c r="C283" s="27" t="n"/>
+      <c r="C283" s="23" t="n"/>
       <c r="D283" s="19" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="18" t="n"/>
       <c r="B284" s="19" t="n"/>
-      <c r="C284" s="27" t="n"/>
+      <c r="C284" s="23" t="n"/>
       <c r="D284" s="19" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="18" t="n"/>
       <c r="B285" s="19" t="n"/>
-      <c r="C285" s="27" t="n"/>
+      <c r="C285" s="23" t="n"/>
       <c r="D285" s="19" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="18" t="n"/>
       <c r="B286" s="19" t="n"/>
-      <c r="C286" s="27" t="n"/>
+      <c r="C286" s="23" t="n"/>
       <c r="D286" s="19" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="18" t="n"/>
       <c r="B287" s="19" t="n"/>
-      <c r="C287" s="27" t="n"/>
+      <c r="C287" s="23" t="n"/>
       <c r="D287" s="19" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="18" t="n"/>
       <c r="B288" s="19" t="n"/>
-      <c r="C288" s="27" t="n"/>
+      <c r="C288" s="23" t="n"/>
       <c r="D288" s="19" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="18" t="n"/>
       <c r="B289" s="19" t="n"/>
-      <c r="C289" s="27" t="n"/>
+      <c r="C289" s="23" t="n"/>
       <c r="D289" s="19" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="18" t="n"/>
       <c r="B290" s="19" t="n"/>
-      <c r="C290" s="27" t="n"/>
+      <c r="C290" s="23" t="n"/>
       <c r="D290" s="19" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="18" t="n"/>
       <c r="B291" s="19" t="n"/>
-      <c r="C291" s="27" t="n"/>
+      <c r="C291" s="23" t="n"/>
       <c r="D291" s="19" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="18" t="n"/>
       <c r="B292" s="19" t="n"/>
-      <c r="C292" s="27" t="n"/>
+      <c r="C292" s="23" t="n"/>
       <c r="D292" s="19" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="18" t="n"/>
       <c r="B293" s="19" t="n"/>
-      <c r="C293" s="27" t="n"/>
+      <c r="C293" s="23" t="n"/>
       <c r="D293" s="19" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="18" t="n"/>
       <c r="B294" s="19" t="n"/>
-      <c r="C294" s="27" t="n"/>
+      <c r="C294" s="23" t="n"/>
       <c r="D294" s="19" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="18" t="n"/>
       <c r="B295" s="19" t="n"/>
-      <c r="C295" s="27" t="n"/>
+      <c r="C295" s="23" t="n"/>
       <c r="D295" s="19" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="18" t="n"/>
       <c r="B296" s="19" t="n"/>
-      <c r="C296" s="27" t="n"/>
+      <c r="C296" s="23" t="n"/>
       <c r="D296" s="19" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="18" t="n"/>
       <c r="B297" s="19" t="n"/>
-      <c r="C297" s="27" t="n"/>
+      <c r="C297" s="23" t="n"/>
       <c r="D297" s="19" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="18" t="n"/>
       <c r="B298" s="19" t="n"/>
-      <c r="C298" s="27" t="n"/>
+      <c r="C298" s="23" t="n"/>
       <c r="D298" s="19" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="18" t="n"/>
       <c r="B299" s="19" t="n"/>
-      <c r="C299" s="27" t="n"/>
+      <c r="C299" s="23" t="n"/>
       <c r="D299" s="19" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="18" t="n"/>
       <c r="B300" s="19" t="n"/>
-      <c r="C300" s="27" t="n"/>
+      <c r="C300" s="23" t="n"/>
       <c r="D300" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="B30:D30"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9285,7 +9187,7 @@
           <t>Obiettivo del fondo (€)</t>
         </is>
       </c>
-      <c r="B3" s="29" t="n">
+      <c r="B3" s="25" t="n">
         <v>5000</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -9300,7 +9202,7 @@
           <t>Accantonamento buffer al mese (€)</t>
         </is>
       </c>
-      <c r="B4" s="29" t="n">
+      <c r="B4" s="25" t="n">
         <v>150</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -9315,7 +9217,7 @@
           <t>Inizio accantonamento buffer</t>
         </is>
       </c>
-      <c r="B5" s="30" t="n">
+      <c r="B5" s="26" t="n">
         <v>46266</v>
       </c>
       <c r="C5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
finanze: Movimenti con importi sempre positivi e colonna Tipo
Il segno meno confondeva le somme fatte a mano. Ora Importo è sempre
positivo e la direzione (spesa/accredito) sta nella colonna Tipo.
</commit_message>
<xml_diff>
--- a/finanze/quaderno-5000.xlsx
+++ b/finanze/quaderno-5000.xlsx
@@ -7029,13 +7029,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D300"/>
+  <dimension ref="A1:E300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="58" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7045,10 +7046,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="42" customHeight="1">
+    <row r="2" ht="50" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Nessuna formula qui dentro: è solo un elenco. Le somme e i confronti li fai tu, come vuoi. Per aggiungere una categoria nuova basta scriverla nella colonna Categoria — non c'è nulla da rompere. Il raggruppamento per data e categoria te lo preparo io in chat ogni volta che incolli i movimenti nuovi: tu li copi qui sotto così come sono.</t>
+          <t>Nessuna formula qui dentro: è solo un elenco. Le somme e i confronti li fai tu, come vuoi. Importo è sempre positivo: la direzione (spesa o accredito) è nella colonna Tipo, così non ti tocca fare i conti con il segno meno. Per aggiungere una categoria nuova basta scriverla — non c'è nulla da rompere. Il raggruppamento per data e categoria te lo preparo io in chat ogni volta che incolli i movimenti nuovi: tu li copi qui sotto così come sono.</t>
         </is>
       </c>
     </row>
@@ -7069,6 +7070,11 @@
         </is>
       </c>
       <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E4" s="20" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
@@ -7088,6 +7094,11 @@
       </c>
       <c r="D5" s="17" t="inlineStr">
         <is>
+          <t>Accredito</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="inlineStr">
+        <is>
           <t>Trasferimento</t>
         </is>
       </c>
@@ -7106,6 +7117,11 @@
       </c>
       <c r="D6" s="17" t="inlineStr">
         <is>
+          <t>Accredito</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
           <t>Entrata</t>
         </is>
       </c>
@@ -7120,9 +7136,14 @@
         </is>
       </c>
       <c r="C7" s="22" t="n">
-        <v>-26.3</v>
+        <v>26.3</v>
       </c>
       <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>Spesa</t>
+        </is>
+      </c>
+      <c r="E7" s="17" t="inlineStr">
         <is>
           <t>Benzina</t>
         </is>
@@ -7138,9 +7159,14 @@
         </is>
       </c>
       <c r="C8" s="22" t="n">
-        <v>-4.14</v>
+        <v>4.14</v>
       </c>
       <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>Spesa</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
         <is>
           <t>Cibo</t>
         </is>
@@ -7156,9 +7182,14 @@
         </is>
       </c>
       <c r="C9" s="22" t="n">
-        <v>-7.57</v>
+        <v>7.57</v>
       </c>
       <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>Spesa</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>Cibo</t>
         </is>
@@ -7174,9 +7205,14 @@
         </is>
       </c>
       <c r="C10" s="22" t="n">
-        <v>-46</v>
+        <v>46</v>
       </c>
       <c r="D10" s="17" t="inlineStr">
+        <is>
+          <t>Spesa</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
         <is>
           <t>Cibo</t>
         </is>
@@ -7192,9 +7228,14 @@
         </is>
       </c>
       <c r="C11" s="22" t="n">
-        <v>-1.5</v>
+        <v>1.5</v>
       </c>
       <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>Spesa</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
         <is>
           <t>Bollette</t>
         </is>
@@ -7210,9 +7251,14 @@
         </is>
       </c>
       <c r="C12" s="22" t="n">
-        <v>-137.49</v>
+        <v>137.49</v>
       </c>
       <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>Spesa</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
         <is>
           <t>Bollette</t>
         </is>
@@ -7228,9 +7274,14 @@
         </is>
       </c>
       <c r="C13" s="22" t="n">
-        <v>-1.5</v>
+        <v>1.5</v>
       </c>
       <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>Spesa</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
         <is>
           <t>Bollette</t>
         </is>
@@ -7246,9 +7297,14 @@
         </is>
       </c>
       <c r="C14" s="22" t="n">
-        <v>-84.76000000000001</v>
+        <v>84.76000000000001</v>
       </c>
       <c r="D14" s="17" t="inlineStr">
+        <is>
+          <t>Spesa</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
         <is>
           <t>Bollette</t>
         </is>
@@ -7264,9 +7320,14 @@
         </is>
       </c>
       <c r="C15" s="22" t="n">
-        <v>-1.95</v>
+        <v>1.95</v>
       </c>
       <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>Spesa</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="inlineStr">
         <is>
           <t>Cibo</t>
         </is>
@@ -7282,9 +7343,14 @@
         </is>
       </c>
       <c r="C16" s="22" t="n">
-        <v>-9</v>
+        <v>9</v>
       </c>
       <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t>Spesa</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
         <is>
           <t>Cibo</t>
         </is>
@@ -7300,9 +7366,14 @@
         </is>
       </c>
       <c r="C17" s="22" t="n">
-        <v>-18</v>
+        <v>18</v>
       </c>
       <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>Spesa</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
         <is>
           <t>Cibo</t>
         </is>
@@ -7318,9 +7389,14 @@
         </is>
       </c>
       <c r="C18" s="22" t="n">
-        <v>-9</v>
+        <v>9</v>
       </c>
       <c r="D18" s="17" t="inlineStr">
+        <is>
+          <t>Spesa</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
         <is>
           <t>Cibo</t>
         </is>
@@ -7336,9 +7412,14 @@
         </is>
       </c>
       <c r="C19" s="22" t="n">
-        <v>-470</v>
+        <v>470</v>
       </c>
       <c r="D19" s="17" t="inlineStr">
+        <is>
+          <t>Spesa</t>
+        </is>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
         <is>
           <t>Trasferimento</t>
         </is>
@@ -7354,9 +7435,14 @@
         </is>
       </c>
       <c r="C20" s="22" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="D20" s="17" t="inlineStr">
+        <is>
+          <t>Spesa</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
         <is>
           <t>Trasferimento</t>
         </is>
@@ -7372,9 +7458,14 @@
         </is>
       </c>
       <c r="C21" s="22" t="n">
-        <v>-25</v>
+        <v>25</v>
       </c>
       <c r="D21" s="17" t="inlineStr">
+        <is>
+          <t>Spesa</t>
+        </is>
+      </c>
+      <c r="E21" s="17" t="inlineStr">
         <is>
           <t>Trasferimento</t>
         </is>
@@ -7390,9 +7481,14 @@
         </is>
       </c>
       <c r="C22" s="22" t="n">
-        <v>-27.84</v>
+        <v>27.84</v>
       </c>
       <c r="D22" s="17" t="inlineStr">
+        <is>
+          <t>Spesa</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="inlineStr">
         <is>
           <t>Benzina</t>
         </is>
@@ -7408,9 +7504,14 @@
         </is>
       </c>
       <c r="C23" s="22" t="n">
-        <v>-1.73</v>
+        <v>1.73</v>
       </c>
       <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>Spesa</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="inlineStr">
         <is>
           <t>Cibo</t>
         </is>
@@ -7426,9 +7527,14 @@
         </is>
       </c>
       <c r="C24" s="22" t="n">
-        <v>-9</v>
+        <v>9</v>
       </c>
       <c r="D24" s="17" t="inlineStr">
+        <is>
+          <t>Spesa</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="inlineStr">
         <is>
           <t>Cibo</t>
         </is>
@@ -7444,9 +7550,14 @@
         </is>
       </c>
       <c r="C25" s="22" t="n">
-        <v>-21.96</v>
+        <v>21.96</v>
       </c>
       <c r="D25" s="17" t="inlineStr">
+        <is>
+          <t>Spesa</t>
+        </is>
+      </c>
+      <c r="E25" s="17" t="inlineStr">
         <is>
           <t>Abbonamenti</t>
         </is>
@@ -7466,6 +7577,11 @@
       </c>
       <c r="D26" s="17" t="inlineStr">
         <is>
+          <t>Accredito</t>
+        </is>
+      </c>
+      <c r="E26" s="17" t="inlineStr">
+        <is>
           <t>Trasferimento</t>
         </is>
       </c>
@@ -7480,9 +7596,14 @@
         </is>
       </c>
       <c r="C27" s="22" t="n">
-        <v>-27</v>
+        <v>27</v>
       </c>
       <c r="D27" s="17" t="inlineStr">
+        <is>
+          <t>Spesa</t>
+        </is>
+      </c>
+      <c r="E27" s="17" t="inlineStr">
         <is>
           <t>Cibo</t>
         </is>
@@ -7498,9 +7619,14 @@
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>-36</v>
+        <v>36</v>
       </c>
       <c r="D28" s="17" t="inlineStr">
+        <is>
+          <t>Spesa</t>
+        </is>
+      </c>
+      <c r="E28" s="17" t="inlineStr">
         <is>
           <t>Cibo</t>
         </is>
@@ -7511,6 +7637,7 @@
       <c r="B29" s="19" t="n"/>
       <c r="C29" s="23" t="n"/>
       <c r="D29" s="19" t="n"/>
+      <c r="E29" s="19" t="n"/>
     </row>
     <row r="30" ht="50" customHeight="1">
       <c r="A30" s="24" t="inlineStr">
@@ -7529,1625 +7656,1895 @@
       <c r="B31" s="19" t="n"/>
       <c r="C31" s="23" t="n"/>
       <c r="D31" s="19" t="n"/>
+      <c r="E31" s="19" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="18" t="n"/>
       <c r="B32" s="19" t="n"/>
       <c r="C32" s="23" t="n"/>
       <c r="D32" s="19" t="n"/>
+      <c r="E32" s="19" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="18" t="n"/>
       <c r="B33" s="19" t="n"/>
       <c r="C33" s="23" t="n"/>
       <c r="D33" s="19" t="n"/>
+      <c r="E33" s="19" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="18" t="n"/>
       <c r="B34" s="19" t="n"/>
       <c r="C34" s="23" t="n"/>
       <c r="D34" s="19" t="n"/>
+      <c r="E34" s="19" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="18" t="n"/>
       <c r="B35" s="19" t="n"/>
       <c r="C35" s="23" t="n"/>
       <c r="D35" s="19" t="n"/>
+      <c r="E35" s="19" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="18" t="n"/>
       <c r="B36" s="19" t="n"/>
       <c r="C36" s="23" t="n"/>
       <c r="D36" s="19" t="n"/>
+      <c r="E36" s="19" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="18" t="n"/>
       <c r="B37" s="19" t="n"/>
       <c r="C37" s="23" t="n"/>
       <c r="D37" s="19" t="n"/>
+      <c r="E37" s="19" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="18" t="n"/>
       <c r="B38" s="19" t="n"/>
       <c r="C38" s="23" t="n"/>
       <c r="D38" s="19" t="n"/>
+      <c r="E38" s="19" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="18" t="n"/>
       <c r="B39" s="19" t="n"/>
       <c r="C39" s="23" t="n"/>
       <c r="D39" s="19" t="n"/>
+      <c r="E39" s="19" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="18" t="n"/>
       <c r="B40" s="19" t="n"/>
       <c r="C40" s="23" t="n"/>
       <c r="D40" s="19" t="n"/>
+      <c r="E40" s="19" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="18" t="n"/>
       <c r="B41" s="19" t="n"/>
       <c r="C41" s="23" t="n"/>
       <c r="D41" s="19" t="n"/>
+      <c r="E41" s="19" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="18" t="n"/>
       <c r="B42" s="19" t="n"/>
       <c r="C42" s="23" t="n"/>
       <c r="D42" s="19" t="n"/>
+      <c r="E42" s="19" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="18" t="n"/>
       <c r="B43" s="19" t="n"/>
       <c r="C43" s="23" t="n"/>
       <c r="D43" s="19" t="n"/>
+      <c r="E43" s="19" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="18" t="n"/>
       <c r="B44" s="19" t="n"/>
       <c r="C44" s="23" t="n"/>
       <c r="D44" s="19" t="n"/>
+      <c r="E44" s="19" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="18" t="n"/>
       <c r="B45" s="19" t="n"/>
       <c r="C45" s="23" t="n"/>
       <c r="D45" s="19" t="n"/>
+      <c r="E45" s="19" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="18" t="n"/>
       <c r="B46" s="19" t="n"/>
       <c r="C46" s="23" t="n"/>
       <c r="D46" s="19" t="n"/>
+      <c r="E46" s="19" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="18" t="n"/>
       <c r="B47" s="19" t="n"/>
       <c r="C47" s="23" t="n"/>
       <c r="D47" s="19" t="n"/>
+      <c r="E47" s="19" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="18" t="n"/>
       <c r="B48" s="19" t="n"/>
       <c r="C48" s="23" t="n"/>
       <c r="D48" s="19" t="n"/>
+      <c r="E48" s="19" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="18" t="n"/>
       <c r="B49" s="19" t="n"/>
       <c r="C49" s="23" t="n"/>
       <c r="D49" s="19" t="n"/>
+      <c r="E49" s="19" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="18" t="n"/>
       <c r="B50" s="19" t="n"/>
       <c r="C50" s="23" t="n"/>
       <c r="D50" s="19" t="n"/>
+      <c r="E50" s="19" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="18" t="n"/>
       <c r="B51" s="19" t="n"/>
       <c r="C51" s="23" t="n"/>
       <c r="D51" s="19" t="n"/>
+      <c r="E51" s="19" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="18" t="n"/>
       <c r="B52" s="19" t="n"/>
       <c r="C52" s="23" t="n"/>
       <c r="D52" s="19" t="n"/>
+      <c r="E52" s="19" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="18" t="n"/>
       <c r="B53" s="19" t="n"/>
       <c r="C53" s="23" t="n"/>
       <c r="D53" s="19" t="n"/>
+      <c r="E53" s="19" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="18" t="n"/>
       <c r="B54" s="19" t="n"/>
       <c r="C54" s="23" t="n"/>
       <c r="D54" s="19" t="n"/>
+      <c r="E54" s="19" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="18" t="n"/>
       <c r="B55" s="19" t="n"/>
       <c r="C55" s="23" t="n"/>
       <c r="D55" s="19" t="n"/>
+      <c r="E55" s="19" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="18" t="n"/>
       <c r="B56" s="19" t="n"/>
       <c r="C56" s="23" t="n"/>
       <c r="D56" s="19" t="n"/>
+      <c r="E56" s="19" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="18" t="n"/>
       <c r="B57" s="19" t="n"/>
       <c r="C57" s="23" t="n"/>
       <c r="D57" s="19" t="n"/>
+      <c r="E57" s="19" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="18" t="n"/>
       <c r="B58" s="19" t="n"/>
       <c r="C58" s="23" t="n"/>
       <c r="D58" s="19" t="n"/>
+      <c r="E58" s="19" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="18" t="n"/>
       <c r="B59" s="19" t="n"/>
       <c r="C59" s="23" t="n"/>
       <c r="D59" s="19" t="n"/>
+      <c r="E59" s="19" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="18" t="n"/>
       <c r="B60" s="19" t="n"/>
       <c r="C60" s="23" t="n"/>
       <c r="D60" s="19" t="n"/>
+      <c r="E60" s="19" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="18" t="n"/>
       <c r="B61" s="19" t="n"/>
       <c r="C61" s="23" t="n"/>
       <c r="D61" s="19" t="n"/>
+      <c r="E61" s="19" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="18" t="n"/>
       <c r="B62" s="19" t="n"/>
       <c r="C62" s="23" t="n"/>
       <c r="D62" s="19" t="n"/>
+      <c r="E62" s="19" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="18" t="n"/>
       <c r="B63" s="19" t="n"/>
       <c r="C63" s="23" t="n"/>
       <c r="D63" s="19" t="n"/>
+      <c r="E63" s="19" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="18" t="n"/>
       <c r="B64" s="19" t="n"/>
       <c r="C64" s="23" t="n"/>
       <c r="D64" s="19" t="n"/>
+      <c r="E64" s="19" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="18" t="n"/>
       <c r="B65" s="19" t="n"/>
       <c r="C65" s="23" t="n"/>
       <c r="D65" s="19" t="n"/>
+      <c r="E65" s="19" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="18" t="n"/>
       <c r="B66" s="19" t="n"/>
       <c r="C66" s="23" t="n"/>
       <c r="D66" s="19" t="n"/>
+      <c r="E66" s="19" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="18" t="n"/>
       <c r="B67" s="19" t="n"/>
       <c r="C67" s="23" t="n"/>
       <c r="D67" s="19" t="n"/>
+      <c r="E67" s="19" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="18" t="n"/>
       <c r="B68" s="19" t="n"/>
       <c r="C68" s="23" t="n"/>
       <c r="D68" s="19" t="n"/>
+      <c r="E68" s="19" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="18" t="n"/>
       <c r="B69" s="19" t="n"/>
       <c r="C69" s="23" t="n"/>
       <c r="D69" s="19" t="n"/>
+      <c r="E69" s="19" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="18" t="n"/>
       <c r="B70" s="19" t="n"/>
       <c r="C70" s="23" t="n"/>
       <c r="D70" s="19" t="n"/>
+      <c r="E70" s="19" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="18" t="n"/>
       <c r="B71" s="19" t="n"/>
       <c r="C71" s="23" t="n"/>
       <c r="D71" s="19" t="n"/>
+      <c r="E71" s="19" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="18" t="n"/>
       <c r="B72" s="19" t="n"/>
       <c r="C72" s="23" t="n"/>
       <c r="D72" s="19" t="n"/>
+      <c r="E72" s="19" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="18" t="n"/>
       <c r="B73" s="19" t="n"/>
       <c r="C73" s="23" t="n"/>
       <c r="D73" s="19" t="n"/>
+      <c r="E73" s="19" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="18" t="n"/>
       <c r="B74" s="19" t="n"/>
       <c r="C74" s="23" t="n"/>
       <c r="D74" s="19" t="n"/>
+      <c r="E74" s="19" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="18" t="n"/>
       <c r="B75" s="19" t="n"/>
       <c r="C75" s="23" t="n"/>
       <c r="D75" s="19" t="n"/>
+      <c r="E75" s="19" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="18" t="n"/>
       <c r="B76" s="19" t="n"/>
       <c r="C76" s="23" t="n"/>
       <c r="D76" s="19" t="n"/>
+      <c r="E76" s="19" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="18" t="n"/>
       <c r="B77" s="19" t="n"/>
       <c r="C77" s="23" t="n"/>
       <c r="D77" s="19" t="n"/>
+      <c r="E77" s="19" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="18" t="n"/>
       <c r="B78" s="19" t="n"/>
       <c r="C78" s="23" t="n"/>
       <c r="D78" s="19" t="n"/>
+      <c r="E78" s="19" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="18" t="n"/>
       <c r="B79" s="19" t="n"/>
       <c r="C79" s="23" t="n"/>
       <c r="D79" s="19" t="n"/>
+      <c r="E79" s="19" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="18" t="n"/>
       <c r="B80" s="19" t="n"/>
       <c r="C80" s="23" t="n"/>
       <c r="D80" s="19" t="n"/>
+      <c r="E80" s="19" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="18" t="n"/>
       <c r="B81" s="19" t="n"/>
       <c r="C81" s="23" t="n"/>
       <c r="D81" s="19" t="n"/>
+      <c r="E81" s="19" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="18" t="n"/>
       <c r="B82" s="19" t="n"/>
       <c r="C82" s="23" t="n"/>
       <c r="D82" s="19" t="n"/>
+      <c r="E82" s="19" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="18" t="n"/>
       <c r="B83" s="19" t="n"/>
       <c r="C83" s="23" t="n"/>
       <c r="D83" s="19" t="n"/>
+      <c r="E83" s="19" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="18" t="n"/>
       <c r="B84" s="19" t="n"/>
       <c r="C84" s="23" t="n"/>
       <c r="D84" s="19" t="n"/>
+      <c r="E84" s="19" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="18" t="n"/>
       <c r="B85" s="19" t="n"/>
       <c r="C85" s="23" t="n"/>
       <c r="D85" s="19" t="n"/>
+      <c r="E85" s="19" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="18" t="n"/>
       <c r="B86" s="19" t="n"/>
       <c r="C86" s="23" t="n"/>
       <c r="D86" s="19" t="n"/>
+      <c r="E86" s="19" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="18" t="n"/>
       <c r="B87" s="19" t="n"/>
       <c r="C87" s="23" t="n"/>
       <c r="D87" s="19" t="n"/>
+      <c r="E87" s="19" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="18" t="n"/>
       <c r="B88" s="19" t="n"/>
       <c r="C88" s="23" t="n"/>
       <c r="D88" s="19" t="n"/>
+      <c r="E88" s="19" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="18" t="n"/>
       <c r="B89" s="19" t="n"/>
       <c r="C89" s="23" t="n"/>
       <c r="D89" s="19" t="n"/>
+      <c r="E89" s="19" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="18" t="n"/>
       <c r="B90" s="19" t="n"/>
       <c r="C90" s="23" t="n"/>
       <c r="D90" s="19" t="n"/>
+      <c r="E90" s="19" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="18" t="n"/>
       <c r="B91" s="19" t="n"/>
       <c r="C91" s="23" t="n"/>
       <c r="D91" s="19" t="n"/>
+      <c r="E91" s="19" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="18" t="n"/>
       <c r="B92" s="19" t="n"/>
       <c r="C92" s="23" t="n"/>
       <c r="D92" s="19" t="n"/>
+      <c r="E92" s="19" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="18" t="n"/>
       <c r="B93" s="19" t="n"/>
       <c r="C93" s="23" t="n"/>
       <c r="D93" s="19" t="n"/>
+      <c r="E93" s="19" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="18" t="n"/>
       <c r="B94" s="19" t="n"/>
       <c r="C94" s="23" t="n"/>
       <c r="D94" s="19" t="n"/>
+      <c r="E94" s="19" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="18" t="n"/>
       <c r="B95" s="19" t="n"/>
       <c r="C95" s="23" t="n"/>
       <c r="D95" s="19" t="n"/>
+      <c r="E95" s="19" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="18" t="n"/>
       <c r="B96" s="19" t="n"/>
       <c r="C96" s="23" t="n"/>
       <c r="D96" s="19" t="n"/>
+      <c r="E96" s="19" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="18" t="n"/>
       <c r="B97" s="19" t="n"/>
       <c r="C97" s="23" t="n"/>
       <c r="D97" s="19" t="n"/>
+      <c r="E97" s="19" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="18" t="n"/>
       <c r="B98" s="19" t="n"/>
       <c r="C98" s="23" t="n"/>
       <c r="D98" s="19" t="n"/>
+      <c r="E98" s="19" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="18" t="n"/>
       <c r="B99" s="19" t="n"/>
       <c r="C99" s="23" t="n"/>
       <c r="D99" s="19" t="n"/>
+      <c r="E99" s="19" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="18" t="n"/>
       <c r="B100" s="19" t="n"/>
       <c r="C100" s="23" t="n"/>
       <c r="D100" s="19" t="n"/>
+      <c r="E100" s="19" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="18" t="n"/>
       <c r="B101" s="19" t="n"/>
       <c r="C101" s="23" t="n"/>
       <c r="D101" s="19" t="n"/>
+      <c r="E101" s="19" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="18" t="n"/>
       <c r="B102" s="19" t="n"/>
       <c r="C102" s="23" t="n"/>
       <c r="D102" s="19" t="n"/>
+      <c r="E102" s="19" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="18" t="n"/>
       <c r="B103" s="19" t="n"/>
       <c r="C103" s="23" t="n"/>
       <c r="D103" s="19" t="n"/>
+      <c r="E103" s="19" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="18" t="n"/>
       <c r="B104" s="19" t="n"/>
       <c r="C104" s="23" t="n"/>
       <c r="D104" s="19" t="n"/>
+      <c r="E104" s="19" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="18" t="n"/>
       <c r="B105" s="19" t="n"/>
       <c r="C105" s="23" t="n"/>
       <c r="D105" s="19" t="n"/>
+      <c r="E105" s="19" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="18" t="n"/>
       <c r="B106" s="19" t="n"/>
       <c r="C106" s="23" t="n"/>
       <c r="D106" s="19" t="n"/>
+      <c r="E106" s="19" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="18" t="n"/>
       <c r="B107" s="19" t="n"/>
       <c r="C107" s="23" t="n"/>
       <c r="D107" s="19" t="n"/>
+      <c r="E107" s="19" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="18" t="n"/>
       <c r="B108" s="19" t="n"/>
       <c r="C108" s="23" t="n"/>
       <c r="D108" s="19" t="n"/>
+      <c r="E108" s="19" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="18" t="n"/>
       <c r="B109" s="19" t="n"/>
       <c r="C109" s="23" t="n"/>
       <c r="D109" s="19" t="n"/>
+      <c r="E109" s="19" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="18" t="n"/>
       <c r="B110" s="19" t="n"/>
       <c r="C110" s="23" t="n"/>
       <c r="D110" s="19" t="n"/>
+      <c r="E110" s="19" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="18" t="n"/>
       <c r="B111" s="19" t="n"/>
       <c r="C111" s="23" t="n"/>
       <c r="D111" s="19" t="n"/>
+      <c r="E111" s="19" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="18" t="n"/>
       <c r="B112" s="19" t="n"/>
       <c r="C112" s="23" t="n"/>
       <c r="D112" s="19" t="n"/>
+      <c r="E112" s="19" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="18" t="n"/>
       <c r="B113" s="19" t="n"/>
       <c r="C113" s="23" t="n"/>
       <c r="D113" s="19" t="n"/>
+      <c r="E113" s="19" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="18" t="n"/>
       <c r="B114" s="19" t="n"/>
       <c r="C114" s="23" t="n"/>
       <c r="D114" s="19" t="n"/>
+      <c r="E114" s="19" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="18" t="n"/>
       <c r="B115" s="19" t="n"/>
       <c r="C115" s="23" t="n"/>
       <c r="D115" s="19" t="n"/>
+      <c r="E115" s="19" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="18" t="n"/>
       <c r="B116" s="19" t="n"/>
       <c r="C116" s="23" t="n"/>
       <c r="D116" s="19" t="n"/>
+      <c r="E116" s="19" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="18" t="n"/>
       <c r="B117" s="19" t="n"/>
       <c r="C117" s="23" t="n"/>
       <c r="D117" s="19" t="n"/>
+      <c r="E117" s="19" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="18" t="n"/>
       <c r="B118" s="19" t="n"/>
       <c r="C118" s="23" t="n"/>
       <c r="D118" s="19" t="n"/>
+      <c r="E118" s="19" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="18" t="n"/>
       <c r="B119" s="19" t="n"/>
       <c r="C119" s="23" t="n"/>
       <c r="D119" s="19" t="n"/>
+      <c r="E119" s="19" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="18" t="n"/>
       <c r="B120" s="19" t="n"/>
       <c r="C120" s="23" t="n"/>
       <c r="D120" s="19" t="n"/>
+      <c r="E120" s="19" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="18" t="n"/>
       <c r="B121" s="19" t="n"/>
       <c r="C121" s="23" t="n"/>
       <c r="D121" s="19" t="n"/>
+      <c r="E121" s="19" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="18" t="n"/>
       <c r="B122" s="19" t="n"/>
       <c r="C122" s="23" t="n"/>
       <c r="D122" s="19" t="n"/>
+      <c r="E122" s="19" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="18" t="n"/>
       <c r="B123" s="19" t="n"/>
       <c r="C123" s="23" t="n"/>
       <c r="D123" s="19" t="n"/>
+      <c r="E123" s="19" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="18" t="n"/>
       <c r="B124" s="19" t="n"/>
       <c r="C124" s="23" t="n"/>
       <c r="D124" s="19" t="n"/>
+      <c r="E124" s="19" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="18" t="n"/>
       <c r="B125" s="19" t="n"/>
       <c r="C125" s="23" t="n"/>
       <c r="D125" s="19" t="n"/>
+      <c r="E125" s="19" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="18" t="n"/>
       <c r="B126" s="19" t="n"/>
       <c r="C126" s="23" t="n"/>
       <c r="D126" s="19" t="n"/>
+      <c r="E126" s="19" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="18" t="n"/>
       <c r="B127" s="19" t="n"/>
       <c r="C127" s="23" t="n"/>
       <c r="D127" s="19" t="n"/>
+      <c r="E127" s="19" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="18" t="n"/>
       <c r="B128" s="19" t="n"/>
       <c r="C128" s="23" t="n"/>
       <c r="D128" s="19" t="n"/>
+      <c r="E128" s="19" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="18" t="n"/>
       <c r="B129" s="19" t="n"/>
       <c r="C129" s="23" t="n"/>
       <c r="D129" s="19" t="n"/>
+      <c r="E129" s="19" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="18" t="n"/>
       <c r="B130" s="19" t="n"/>
       <c r="C130" s="23" t="n"/>
       <c r="D130" s="19" t="n"/>
+      <c r="E130" s="19" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="18" t="n"/>
       <c r="B131" s="19" t="n"/>
       <c r="C131" s="23" t="n"/>
       <c r="D131" s="19" t="n"/>
+      <c r="E131" s="19" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="18" t="n"/>
       <c r="B132" s="19" t="n"/>
       <c r="C132" s="23" t="n"/>
       <c r="D132" s="19" t="n"/>
+      <c r="E132" s="19" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="18" t="n"/>
       <c r="B133" s="19" t="n"/>
       <c r="C133" s="23" t="n"/>
       <c r="D133" s="19" t="n"/>
+      <c r="E133" s="19" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="18" t="n"/>
       <c r="B134" s="19" t="n"/>
       <c r="C134" s="23" t="n"/>
       <c r="D134" s="19" t="n"/>
+      <c r="E134" s="19" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="18" t="n"/>
       <c r="B135" s="19" t="n"/>
       <c r="C135" s="23" t="n"/>
       <c r="D135" s="19" t="n"/>
+      <c r="E135" s="19" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="18" t="n"/>
       <c r="B136" s="19" t="n"/>
       <c r="C136" s="23" t="n"/>
       <c r="D136" s="19" t="n"/>
+      <c r="E136" s="19" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="18" t="n"/>
       <c r="B137" s="19" t="n"/>
       <c r="C137" s="23" t="n"/>
       <c r="D137" s="19" t="n"/>
+      <c r="E137" s="19" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="18" t="n"/>
       <c r="B138" s="19" t="n"/>
       <c r="C138" s="23" t="n"/>
       <c r="D138" s="19" t="n"/>
+      <c r="E138" s="19" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="18" t="n"/>
       <c r="B139" s="19" t="n"/>
       <c r="C139" s="23" t="n"/>
       <c r="D139" s="19" t="n"/>
+      <c r="E139" s="19" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="18" t="n"/>
       <c r="B140" s="19" t="n"/>
       <c r="C140" s="23" t="n"/>
       <c r="D140" s="19" t="n"/>
+      <c r="E140" s="19" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="18" t="n"/>
       <c r="B141" s="19" t="n"/>
       <c r="C141" s="23" t="n"/>
       <c r="D141" s="19" t="n"/>
+      <c r="E141" s="19" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="18" t="n"/>
       <c r="B142" s="19" t="n"/>
       <c r="C142" s="23" t="n"/>
       <c r="D142" s="19" t="n"/>
+      <c r="E142" s="19" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="18" t="n"/>
       <c r="B143" s="19" t="n"/>
       <c r="C143" s="23" t="n"/>
       <c r="D143" s="19" t="n"/>
+      <c r="E143" s="19" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="18" t="n"/>
       <c r="B144" s="19" t="n"/>
       <c r="C144" s="23" t="n"/>
       <c r="D144" s="19" t="n"/>
+      <c r="E144" s="19" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="18" t="n"/>
       <c r="B145" s="19" t="n"/>
       <c r="C145" s="23" t="n"/>
       <c r="D145" s="19" t="n"/>
+      <c r="E145" s="19" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="18" t="n"/>
       <c r="B146" s="19" t="n"/>
       <c r="C146" s="23" t="n"/>
       <c r="D146" s="19" t="n"/>
+      <c r="E146" s="19" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="18" t="n"/>
       <c r="B147" s="19" t="n"/>
       <c r="C147" s="23" t="n"/>
       <c r="D147" s="19" t="n"/>
+      <c r="E147" s="19" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="18" t="n"/>
       <c r="B148" s="19" t="n"/>
       <c r="C148" s="23" t="n"/>
       <c r="D148" s="19" t="n"/>
+      <c r="E148" s="19" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="18" t="n"/>
       <c r="B149" s="19" t="n"/>
       <c r="C149" s="23" t="n"/>
       <c r="D149" s="19" t="n"/>
+      <c r="E149" s="19" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="18" t="n"/>
       <c r="B150" s="19" t="n"/>
       <c r="C150" s="23" t="n"/>
       <c r="D150" s="19" t="n"/>
+      <c r="E150" s="19" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="18" t="n"/>
       <c r="B151" s="19" t="n"/>
       <c r="C151" s="23" t="n"/>
       <c r="D151" s="19" t="n"/>
+      <c r="E151" s="19" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="18" t="n"/>
       <c r="B152" s="19" t="n"/>
       <c r="C152" s="23" t="n"/>
       <c r="D152" s="19" t="n"/>
+      <c r="E152" s="19" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="18" t="n"/>
       <c r="B153" s="19" t="n"/>
       <c r="C153" s="23" t="n"/>
       <c r="D153" s="19" t="n"/>
+      <c r="E153" s="19" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="18" t="n"/>
       <c r="B154" s="19" t="n"/>
       <c r="C154" s="23" t="n"/>
       <c r="D154" s="19" t="n"/>
+      <c r="E154" s="19" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="18" t="n"/>
       <c r="B155" s="19" t="n"/>
       <c r="C155" s="23" t="n"/>
       <c r="D155" s="19" t="n"/>
+      <c r="E155" s="19" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="18" t="n"/>
       <c r="B156" s="19" t="n"/>
       <c r="C156" s="23" t="n"/>
       <c r="D156" s="19" t="n"/>
+      <c r="E156" s="19" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="18" t="n"/>
       <c r="B157" s="19" t="n"/>
       <c r="C157" s="23" t="n"/>
       <c r="D157" s="19" t="n"/>
+      <c r="E157" s="19" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="18" t="n"/>
       <c r="B158" s="19" t="n"/>
       <c r="C158" s="23" t="n"/>
       <c r="D158" s="19" t="n"/>
+      <c r="E158" s="19" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="18" t="n"/>
       <c r="B159" s="19" t="n"/>
       <c r="C159" s="23" t="n"/>
       <c r="D159" s="19" t="n"/>
+      <c r="E159" s="19" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="18" t="n"/>
       <c r="B160" s="19" t="n"/>
       <c r="C160" s="23" t="n"/>
       <c r="D160" s="19" t="n"/>
+      <c r="E160" s="19" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="18" t="n"/>
       <c r="B161" s="19" t="n"/>
       <c r="C161" s="23" t="n"/>
       <c r="D161" s="19" t="n"/>
+      <c r="E161" s="19" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="18" t="n"/>
       <c r="B162" s="19" t="n"/>
       <c r="C162" s="23" t="n"/>
       <c r="D162" s="19" t="n"/>
+      <c r="E162" s="19" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="18" t="n"/>
       <c r="B163" s="19" t="n"/>
       <c r="C163" s="23" t="n"/>
       <c r="D163" s="19" t="n"/>
+      <c r="E163" s="19" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="18" t="n"/>
       <c r="B164" s="19" t="n"/>
       <c r="C164" s="23" t="n"/>
       <c r="D164" s="19" t="n"/>
+      <c r="E164" s="19" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="18" t="n"/>
       <c r="B165" s="19" t="n"/>
       <c r="C165" s="23" t="n"/>
       <c r="D165" s="19" t="n"/>
+      <c r="E165" s="19" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="18" t="n"/>
       <c r="B166" s="19" t="n"/>
       <c r="C166" s="23" t="n"/>
       <c r="D166" s="19" t="n"/>
+      <c r="E166" s="19" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="18" t="n"/>
       <c r="B167" s="19" t="n"/>
       <c r="C167" s="23" t="n"/>
       <c r="D167" s="19" t="n"/>
+      <c r="E167" s="19" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="18" t="n"/>
       <c r="B168" s="19" t="n"/>
       <c r="C168" s="23" t="n"/>
       <c r="D168" s="19" t="n"/>
+      <c r="E168" s="19" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="18" t="n"/>
       <c r="B169" s="19" t="n"/>
       <c r="C169" s="23" t="n"/>
       <c r="D169" s="19" t="n"/>
+      <c r="E169" s="19" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="18" t="n"/>
       <c r="B170" s="19" t="n"/>
       <c r="C170" s="23" t="n"/>
       <c r="D170" s="19" t="n"/>
+      <c r="E170" s="19" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="18" t="n"/>
       <c r="B171" s="19" t="n"/>
       <c r="C171" s="23" t="n"/>
       <c r="D171" s="19" t="n"/>
+      <c r="E171" s="19" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="18" t="n"/>
       <c r="B172" s="19" t="n"/>
       <c r="C172" s="23" t="n"/>
       <c r="D172" s="19" t="n"/>
+      <c r="E172" s="19" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="18" t="n"/>
       <c r="B173" s="19" t="n"/>
       <c r="C173" s="23" t="n"/>
       <c r="D173" s="19" t="n"/>
+      <c r="E173" s="19" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="18" t="n"/>
       <c r="B174" s="19" t="n"/>
       <c r="C174" s="23" t="n"/>
       <c r="D174" s="19" t="n"/>
+      <c r="E174" s="19" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="18" t="n"/>
       <c r="B175" s="19" t="n"/>
       <c r="C175" s="23" t="n"/>
       <c r="D175" s="19" t="n"/>
+      <c r="E175" s="19" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="18" t="n"/>
       <c r="B176" s="19" t="n"/>
       <c r="C176" s="23" t="n"/>
       <c r="D176" s="19" t="n"/>
+      <c r="E176" s="19" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="18" t="n"/>
       <c r="B177" s="19" t="n"/>
       <c r="C177" s="23" t="n"/>
       <c r="D177" s="19" t="n"/>
+      <c r="E177" s="19" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="18" t="n"/>
       <c r="B178" s="19" t="n"/>
       <c r="C178" s="23" t="n"/>
       <c r="D178" s="19" t="n"/>
+      <c r="E178" s="19" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="18" t="n"/>
       <c r="B179" s="19" t="n"/>
       <c r="C179" s="23" t="n"/>
       <c r="D179" s="19" t="n"/>
+      <c r="E179" s="19" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="18" t="n"/>
       <c r="B180" s="19" t="n"/>
       <c r="C180" s="23" t="n"/>
       <c r="D180" s="19" t="n"/>
+      <c r="E180" s="19" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="18" t="n"/>
       <c r="B181" s="19" t="n"/>
       <c r="C181" s="23" t="n"/>
       <c r="D181" s="19" t="n"/>
+      <c r="E181" s="19" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="18" t="n"/>
       <c r="B182" s="19" t="n"/>
       <c r="C182" s="23" t="n"/>
       <c r="D182" s="19" t="n"/>
+      <c r="E182" s="19" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="18" t="n"/>
       <c r="B183" s="19" t="n"/>
       <c r="C183" s="23" t="n"/>
       <c r="D183" s="19" t="n"/>
+      <c r="E183" s="19" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="18" t="n"/>
       <c r="B184" s="19" t="n"/>
       <c r="C184" s="23" t="n"/>
       <c r="D184" s="19" t="n"/>
+      <c r="E184" s="19" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="18" t="n"/>
       <c r="B185" s="19" t="n"/>
       <c r="C185" s="23" t="n"/>
       <c r="D185" s="19" t="n"/>
+      <c r="E185" s="19" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="18" t="n"/>
       <c r="B186" s="19" t="n"/>
       <c r="C186" s="23" t="n"/>
       <c r="D186" s="19" t="n"/>
+      <c r="E186" s="19" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="18" t="n"/>
       <c r="B187" s="19" t="n"/>
       <c r="C187" s="23" t="n"/>
       <c r="D187" s="19" t="n"/>
+      <c r="E187" s="19" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="18" t="n"/>
       <c r="B188" s="19" t="n"/>
       <c r="C188" s="23" t="n"/>
       <c r="D188" s="19" t="n"/>
+      <c r="E188" s="19" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="18" t="n"/>
       <c r="B189" s="19" t="n"/>
       <c r="C189" s="23" t="n"/>
       <c r="D189" s="19" t="n"/>
+      <c r="E189" s="19" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="18" t="n"/>
       <c r="B190" s="19" t="n"/>
       <c r="C190" s="23" t="n"/>
       <c r="D190" s="19" t="n"/>
+      <c r="E190" s="19" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="18" t="n"/>
       <c r="B191" s="19" t="n"/>
       <c r="C191" s="23" t="n"/>
       <c r="D191" s="19" t="n"/>
+      <c r="E191" s="19" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="18" t="n"/>
       <c r="B192" s="19" t="n"/>
       <c r="C192" s="23" t="n"/>
       <c r="D192" s="19" t="n"/>
+      <c r="E192" s="19" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="18" t="n"/>
       <c r="B193" s="19" t="n"/>
       <c r="C193" s="23" t="n"/>
       <c r="D193" s="19" t="n"/>
+      <c r="E193" s="19" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="18" t="n"/>
       <c r="B194" s="19" t="n"/>
       <c r="C194" s="23" t="n"/>
       <c r="D194" s="19" t="n"/>
+      <c r="E194" s="19" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="18" t="n"/>
       <c r="B195" s="19" t="n"/>
       <c r="C195" s="23" t="n"/>
       <c r="D195" s="19" t="n"/>
+      <c r="E195" s="19" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="18" t="n"/>
       <c r="B196" s="19" t="n"/>
       <c r="C196" s="23" t="n"/>
       <c r="D196" s="19" t="n"/>
+      <c r="E196" s="19" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="18" t="n"/>
       <c r="B197" s="19" t="n"/>
       <c r="C197" s="23" t="n"/>
       <c r="D197" s="19" t="n"/>
+      <c r="E197" s="19" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="18" t="n"/>
       <c r="B198" s="19" t="n"/>
       <c r="C198" s="23" t="n"/>
       <c r="D198" s="19" t="n"/>
+      <c r="E198" s="19" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="18" t="n"/>
       <c r="B199" s="19" t="n"/>
       <c r="C199" s="23" t="n"/>
       <c r="D199" s="19" t="n"/>
+      <c r="E199" s="19" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="18" t="n"/>
       <c r="B200" s="19" t="n"/>
       <c r="C200" s="23" t="n"/>
       <c r="D200" s="19" t="n"/>
+      <c r="E200" s="19" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="18" t="n"/>
       <c r="B201" s="19" t="n"/>
       <c r="C201" s="23" t="n"/>
       <c r="D201" s="19" t="n"/>
+      <c r="E201" s="19" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="18" t="n"/>
       <c r="B202" s="19" t="n"/>
       <c r="C202" s="23" t="n"/>
       <c r="D202" s="19" t="n"/>
+      <c r="E202" s="19" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="18" t="n"/>
       <c r="B203" s="19" t="n"/>
       <c r="C203" s="23" t="n"/>
       <c r="D203" s="19" t="n"/>
+      <c r="E203" s="19" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="18" t="n"/>
       <c r="B204" s="19" t="n"/>
       <c r="C204" s="23" t="n"/>
       <c r="D204" s="19" t="n"/>
+      <c r="E204" s="19" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="18" t="n"/>
       <c r="B205" s="19" t="n"/>
       <c r="C205" s="23" t="n"/>
       <c r="D205" s="19" t="n"/>
+      <c r="E205" s="19" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="18" t="n"/>
       <c r="B206" s="19" t="n"/>
       <c r="C206" s="23" t="n"/>
       <c r="D206" s="19" t="n"/>
+      <c r="E206" s="19" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="18" t="n"/>
       <c r="B207" s="19" t="n"/>
       <c r="C207" s="23" t="n"/>
       <c r="D207" s="19" t="n"/>
+      <c r="E207" s="19" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="18" t="n"/>
       <c r="B208" s="19" t="n"/>
       <c r="C208" s="23" t="n"/>
       <c r="D208" s="19" t="n"/>
+      <c r="E208" s="19" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="18" t="n"/>
       <c r="B209" s="19" t="n"/>
       <c r="C209" s="23" t="n"/>
       <c r="D209" s="19" t="n"/>
+      <c r="E209" s="19" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="18" t="n"/>
       <c r="B210" s="19" t="n"/>
       <c r="C210" s="23" t="n"/>
       <c r="D210" s="19" t="n"/>
+      <c r="E210" s="19" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="18" t="n"/>
       <c r="B211" s="19" t="n"/>
       <c r="C211" s="23" t="n"/>
       <c r="D211" s="19" t="n"/>
+      <c r="E211" s="19" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="18" t="n"/>
       <c r="B212" s="19" t="n"/>
       <c r="C212" s="23" t="n"/>
       <c r="D212" s="19" t="n"/>
+      <c r="E212" s="19" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="18" t="n"/>
       <c r="B213" s="19" t="n"/>
       <c r="C213" s="23" t="n"/>
       <c r="D213" s="19" t="n"/>
+      <c r="E213" s="19" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="18" t="n"/>
       <c r="B214" s="19" t="n"/>
       <c r="C214" s="23" t="n"/>
       <c r="D214" s="19" t="n"/>
+      <c r="E214" s="19" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="18" t="n"/>
       <c r="B215" s="19" t="n"/>
       <c r="C215" s="23" t="n"/>
       <c r="D215" s="19" t="n"/>
+      <c r="E215" s="19" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="18" t="n"/>
       <c r="B216" s="19" t="n"/>
       <c r="C216" s="23" t="n"/>
       <c r="D216" s="19" t="n"/>
+      <c r="E216" s="19" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="18" t="n"/>
       <c r="B217" s="19" t="n"/>
       <c r="C217" s="23" t="n"/>
       <c r="D217" s="19" t="n"/>
+      <c r="E217" s="19" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="18" t="n"/>
       <c r="B218" s="19" t="n"/>
       <c r="C218" s="23" t="n"/>
       <c r="D218" s="19" t="n"/>
+      <c r="E218" s="19" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="18" t="n"/>
       <c r="B219" s="19" t="n"/>
       <c r="C219" s="23" t="n"/>
       <c r="D219" s="19" t="n"/>
+      <c r="E219" s="19" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="18" t="n"/>
       <c r="B220" s="19" t="n"/>
       <c r="C220" s="23" t="n"/>
       <c r="D220" s="19" t="n"/>
+      <c r="E220" s="19" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="18" t="n"/>
       <c r="B221" s="19" t="n"/>
       <c r="C221" s="23" t="n"/>
       <c r="D221" s="19" t="n"/>
+      <c r="E221" s="19" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="18" t="n"/>
       <c r="B222" s="19" t="n"/>
       <c r="C222" s="23" t="n"/>
       <c r="D222" s="19" t="n"/>
+      <c r="E222" s="19" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="18" t="n"/>
       <c r="B223" s="19" t="n"/>
       <c r="C223" s="23" t="n"/>
       <c r="D223" s="19" t="n"/>
+      <c r="E223" s="19" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="18" t="n"/>
       <c r="B224" s="19" t="n"/>
       <c r="C224" s="23" t="n"/>
       <c r="D224" s="19" t="n"/>
+      <c r="E224" s="19" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="18" t="n"/>
       <c r="B225" s="19" t="n"/>
       <c r="C225" s="23" t="n"/>
       <c r="D225" s="19" t="n"/>
+      <c r="E225" s="19" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="18" t="n"/>
       <c r="B226" s="19" t="n"/>
       <c r="C226" s="23" t="n"/>
       <c r="D226" s="19" t="n"/>
+      <c r="E226" s="19" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="18" t="n"/>
       <c r="B227" s="19" t="n"/>
       <c r="C227" s="23" t="n"/>
       <c r="D227" s="19" t="n"/>
+      <c r="E227" s="19" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="18" t="n"/>
       <c r="B228" s="19" t="n"/>
       <c r="C228" s="23" t="n"/>
       <c r="D228" s="19" t="n"/>
+      <c r="E228" s="19" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="18" t="n"/>
       <c r="B229" s="19" t="n"/>
       <c r="C229" s="23" t="n"/>
       <c r="D229" s="19" t="n"/>
+      <c r="E229" s="19" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="18" t="n"/>
       <c r="B230" s="19" t="n"/>
       <c r="C230" s="23" t="n"/>
       <c r="D230" s="19" t="n"/>
+      <c r="E230" s="19" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="18" t="n"/>
       <c r="B231" s="19" t="n"/>
       <c r="C231" s="23" t="n"/>
       <c r="D231" s="19" t="n"/>
+      <c r="E231" s="19" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="18" t="n"/>
       <c r="B232" s="19" t="n"/>
       <c r="C232" s="23" t="n"/>
       <c r="D232" s="19" t="n"/>
+      <c r="E232" s="19" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="18" t="n"/>
       <c r="B233" s="19" t="n"/>
       <c r="C233" s="23" t="n"/>
       <c r="D233" s="19" t="n"/>
+      <c r="E233" s="19" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="18" t="n"/>
       <c r="B234" s="19" t="n"/>
       <c r="C234" s="23" t="n"/>
       <c r="D234" s="19" t="n"/>
+      <c r="E234" s="19" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="18" t="n"/>
       <c r="B235" s="19" t="n"/>
       <c r="C235" s="23" t="n"/>
       <c r="D235" s="19" t="n"/>
+      <c r="E235" s="19" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="18" t="n"/>
       <c r="B236" s="19" t="n"/>
       <c r="C236" s="23" t="n"/>
       <c r="D236" s="19" t="n"/>
+      <c r="E236" s="19" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="18" t="n"/>
       <c r="B237" s="19" t="n"/>
       <c r="C237" s="23" t="n"/>
       <c r="D237" s="19" t="n"/>
+      <c r="E237" s="19" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="18" t="n"/>
       <c r="B238" s="19" t="n"/>
       <c r="C238" s="23" t="n"/>
       <c r="D238" s="19" t="n"/>
+      <c r="E238" s="19" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="18" t="n"/>
       <c r="B239" s="19" t="n"/>
       <c r="C239" s="23" t="n"/>
       <c r="D239" s="19" t="n"/>
+      <c r="E239" s="19" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="18" t="n"/>
       <c r="B240" s="19" t="n"/>
       <c r="C240" s="23" t="n"/>
       <c r="D240" s="19" t="n"/>
+      <c r="E240" s="19" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="18" t="n"/>
       <c r="B241" s="19" t="n"/>
       <c r="C241" s="23" t="n"/>
       <c r="D241" s="19" t="n"/>
+      <c r="E241" s="19" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="18" t="n"/>
       <c r="B242" s="19" t="n"/>
       <c r="C242" s="23" t="n"/>
       <c r="D242" s="19" t="n"/>
+      <c r="E242" s="19" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="18" t="n"/>
       <c r="B243" s="19" t="n"/>
       <c r="C243" s="23" t="n"/>
       <c r="D243" s="19" t="n"/>
+      <c r="E243" s="19" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="18" t="n"/>
       <c r="B244" s="19" t="n"/>
       <c r="C244" s="23" t="n"/>
       <c r="D244" s="19" t="n"/>
+      <c r="E244" s="19" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="18" t="n"/>
       <c r="B245" s="19" t="n"/>
       <c r="C245" s="23" t="n"/>
       <c r="D245" s="19" t="n"/>
+      <c r="E245" s="19" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="18" t="n"/>
       <c r="B246" s="19" t="n"/>
       <c r="C246" s="23" t="n"/>
       <c r="D246" s="19" t="n"/>
+      <c r="E246" s="19" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="18" t="n"/>
       <c r="B247" s="19" t="n"/>
       <c r="C247" s="23" t="n"/>
       <c r="D247" s="19" t="n"/>
+      <c r="E247" s="19" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="18" t="n"/>
       <c r="B248" s="19" t="n"/>
       <c r="C248" s="23" t="n"/>
       <c r="D248" s="19" t="n"/>
+      <c r="E248" s="19" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="18" t="n"/>
       <c r="B249" s="19" t="n"/>
       <c r="C249" s="23" t="n"/>
       <c r="D249" s="19" t="n"/>
+      <c r="E249" s="19" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="18" t="n"/>
       <c r="B250" s="19" t="n"/>
       <c r="C250" s="23" t="n"/>
       <c r="D250" s="19" t="n"/>
+      <c r="E250" s="19" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="18" t="n"/>
       <c r="B251" s="19" t="n"/>
       <c r="C251" s="23" t="n"/>
       <c r="D251" s="19" t="n"/>
+      <c r="E251" s="19" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="18" t="n"/>
       <c r="B252" s="19" t="n"/>
       <c r="C252" s="23" t="n"/>
       <c r="D252" s="19" t="n"/>
+      <c r="E252" s="19" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="18" t="n"/>
       <c r="B253" s="19" t="n"/>
       <c r="C253" s="23" t="n"/>
       <c r="D253" s="19" t="n"/>
+      <c r="E253" s="19" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="18" t="n"/>
       <c r="B254" s="19" t="n"/>
       <c r="C254" s="23" t="n"/>
       <c r="D254" s="19" t="n"/>
+      <c r="E254" s="19" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="18" t="n"/>
       <c r="B255" s="19" t="n"/>
       <c r="C255" s="23" t="n"/>
       <c r="D255" s="19" t="n"/>
+      <c r="E255" s="19" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="18" t="n"/>
       <c r="B256" s="19" t="n"/>
       <c r="C256" s="23" t="n"/>
       <c r="D256" s="19" t="n"/>
+      <c r="E256" s="19" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="18" t="n"/>
       <c r="B257" s="19" t="n"/>
       <c r="C257" s="23" t="n"/>
       <c r="D257" s="19" t="n"/>
+      <c r="E257" s="19" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="18" t="n"/>
       <c r="B258" s="19" t="n"/>
       <c r="C258" s="23" t="n"/>
       <c r="D258" s="19" t="n"/>
+      <c r="E258" s="19" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="18" t="n"/>
       <c r="B259" s="19" t="n"/>
       <c r="C259" s="23" t="n"/>
       <c r="D259" s="19" t="n"/>
+      <c r="E259" s="19" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="18" t="n"/>
       <c r="B260" s="19" t="n"/>
       <c r="C260" s="23" t="n"/>
       <c r="D260" s="19" t="n"/>
+      <c r="E260" s="19" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="18" t="n"/>
       <c r="B261" s="19" t="n"/>
       <c r="C261" s="23" t="n"/>
       <c r="D261" s="19" t="n"/>
+      <c r="E261" s="19" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="18" t="n"/>
       <c r="B262" s="19" t="n"/>
       <c r="C262" s="23" t="n"/>
       <c r="D262" s="19" t="n"/>
+      <c r="E262" s="19" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="18" t="n"/>
       <c r="B263" s="19" t="n"/>
       <c r="C263" s="23" t="n"/>
       <c r="D263" s="19" t="n"/>
+      <c r="E263" s="19" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="18" t="n"/>
       <c r="B264" s="19" t="n"/>
       <c r="C264" s="23" t="n"/>
       <c r="D264" s="19" t="n"/>
+      <c r="E264" s="19" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="18" t="n"/>
       <c r="B265" s="19" t="n"/>
       <c r="C265" s="23" t="n"/>
       <c r="D265" s="19" t="n"/>
+      <c r="E265" s="19" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="18" t="n"/>
       <c r="B266" s="19" t="n"/>
       <c r="C266" s="23" t="n"/>
       <c r="D266" s="19" t="n"/>
+      <c r="E266" s="19" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="18" t="n"/>
       <c r="B267" s="19" t="n"/>
       <c r="C267" s="23" t="n"/>
       <c r="D267" s="19" t="n"/>
+      <c r="E267" s="19" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="18" t="n"/>
       <c r="B268" s="19" t="n"/>
       <c r="C268" s="23" t="n"/>
       <c r="D268" s="19" t="n"/>
+      <c r="E268" s="19" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="18" t="n"/>
       <c r="B269" s="19" t="n"/>
       <c r="C269" s="23" t="n"/>
       <c r="D269" s="19" t="n"/>
+      <c r="E269" s="19" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="18" t="n"/>
       <c r="B270" s="19" t="n"/>
       <c r="C270" s="23" t="n"/>
       <c r="D270" s="19" t="n"/>
+      <c r="E270" s="19" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="18" t="n"/>
       <c r="B271" s="19" t="n"/>
       <c r="C271" s="23" t="n"/>
       <c r="D271" s="19" t="n"/>
+      <c r="E271" s="19" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="18" t="n"/>
       <c r="B272" s="19" t="n"/>
       <c r="C272" s="23" t="n"/>
       <c r="D272" s="19" t="n"/>
+      <c r="E272" s="19" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="18" t="n"/>
       <c r="B273" s="19" t="n"/>
       <c r="C273" s="23" t="n"/>
       <c r="D273" s="19" t="n"/>
+      <c r="E273" s="19" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="18" t="n"/>
       <c r="B274" s="19" t="n"/>
       <c r="C274" s="23" t="n"/>
       <c r="D274" s="19" t="n"/>
+      <c r="E274" s="19" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="18" t="n"/>
       <c r="B275" s="19" t="n"/>
       <c r="C275" s="23" t="n"/>
       <c r="D275" s="19" t="n"/>
+      <c r="E275" s="19" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="18" t="n"/>
       <c r="B276" s="19" t="n"/>
       <c r="C276" s="23" t="n"/>
       <c r="D276" s="19" t="n"/>
+      <c r="E276" s="19" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="18" t="n"/>
       <c r="B277" s="19" t="n"/>
       <c r="C277" s="23" t="n"/>
       <c r="D277" s="19" t="n"/>
+      <c r="E277" s="19" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="18" t="n"/>
       <c r="B278" s="19" t="n"/>
       <c r="C278" s="23" t="n"/>
       <c r="D278" s="19" t="n"/>
+      <c r="E278" s="19" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="18" t="n"/>
       <c r="B279" s="19" t="n"/>
       <c r="C279" s="23" t="n"/>
       <c r="D279" s="19" t="n"/>
+      <c r="E279" s="19" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="18" t="n"/>
       <c r="B280" s="19" t="n"/>
       <c r="C280" s="23" t="n"/>
       <c r="D280" s="19" t="n"/>
+      <c r="E280" s="19" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="18" t="n"/>
       <c r="B281" s="19" t="n"/>
       <c r="C281" s="23" t="n"/>
       <c r="D281" s="19" t="n"/>
+      <c r="E281" s="19" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="18" t="n"/>
       <c r="B282" s="19" t="n"/>
       <c r="C282" s="23" t="n"/>
       <c r="D282" s="19" t="n"/>
+      <c r="E282" s="19" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="18" t="n"/>
       <c r="B283" s="19" t="n"/>
       <c r="C283" s="23" t="n"/>
       <c r="D283" s="19" t="n"/>
+      <c r="E283" s="19" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="18" t="n"/>
       <c r="B284" s="19" t="n"/>
       <c r="C284" s="23" t="n"/>
       <c r="D284" s="19" t="n"/>
+      <c r="E284" s="19" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="18" t="n"/>
       <c r="B285" s="19" t="n"/>
       <c r="C285" s="23" t="n"/>
       <c r="D285" s="19" t="n"/>
+      <c r="E285" s="19" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="18" t="n"/>
       <c r="B286" s="19" t="n"/>
       <c r="C286" s="23" t="n"/>
       <c r="D286" s="19" t="n"/>
+      <c r="E286" s="19" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="18" t="n"/>
       <c r="B287" s="19" t="n"/>
       <c r="C287" s="23" t="n"/>
       <c r="D287" s="19" t="n"/>
+      <c r="E287" s="19" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="18" t="n"/>
       <c r="B288" s="19" t="n"/>
       <c r="C288" s="23" t="n"/>
       <c r="D288" s="19" t="n"/>
+      <c r="E288" s="19" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="18" t="n"/>
       <c r="B289" s="19" t="n"/>
       <c r="C289" s="23" t="n"/>
       <c r="D289" s="19" t="n"/>
+      <c r="E289" s="19" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="18" t="n"/>
       <c r="B290" s="19" t="n"/>
       <c r="C290" s="23" t="n"/>
       <c r="D290" s="19" t="n"/>
+      <c r="E290" s="19" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="18" t="n"/>
       <c r="B291" s="19" t="n"/>
       <c r="C291" s="23" t="n"/>
       <c r="D291" s="19" t="n"/>
+      <c r="E291" s="19" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="18" t="n"/>
       <c r="B292" s="19" t="n"/>
       <c r="C292" s="23" t="n"/>
       <c r="D292" s="19" t="n"/>
+      <c r="E292" s="19" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="18" t="n"/>
       <c r="B293" s="19" t="n"/>
       <c r="C293" s="23" t="n"/>
       <c r="D293" s="19" t="n"/>
+      <c r="E293" s="19" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="18" t="n"/>
       <c r="B294" s="19" t="n"/>
       <c r="C294" s="23" t="n"/>
       <c r="D294" s="19" t="n"/>
+      <c r="E294" s="19" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="18" t="n"/>
       <c r="B295" s="19" t="n"/>
       <c r="C295" s="23" t="n"/>
       <c r="D295" s="19" t="n"/>
+      <c r="E295" s="19" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="18" t="n"/>
       <c r="B296" s="19" t="n"/>
       <c r="C296" s="23" t="n"/>
       <c r="D296" s="19" t="n"/>
+      <c r="E296" s="19" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="18" t="n"/>
       <c r="B297" s="19" t="n"/>
       <c r="C297" s="23" t="n"/>
       <c r="D297" s="19" t="n"/>
+      <c r="E297" s="19" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="18" t="n"/>
       <c r="B298" s="19" t="n"/>
       <c r="C298" s="23" t="n"/>
       <c r="D298" s="19" t="n"/>
+      <c r="E298" s="19" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="18" t="n"/>
       <c r="B299" s="19" t="n"/>
       <c r="C299" s="23" t="n"/>
       <c r="D299" s="19" t="n"/>
+      <c r="E299" s="19" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="18" t="n"/>
       <c r="B300" s="19" t="n"/>
       <c r="C300" s="23" t="n"/>
       <c r="D300" s="19" t="n"/>
+      <c r="E300" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="B30:E30"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
finanze: rifà la curva del Piano, i vecchi numeri non erano aggiornati
La curva precedente (446/1442/2188/4094...) non era stata ricalcolata
dopo aver saputo i costi reali di caldaia, assicurazione e lotta, e le
note contavano la lotta come rata mensile mentre è un pagamento
semestrale unico (nessuna rata fino a marzo). Curva ridotta ai soli
punti verificabili: 20/09 reale (470 €) e 31/10 stimato sul versamento
di 550 € deciso in chat (1.020 €). Da novembre in poi resta esplicitamente
da definire finché non arrivano i dati reali, invece di essere inventata.
</commit_message>
<xml_diff>
--- a/finanze/quaderno-5000.xlsx
+++ b/finanze/quaderno-5000.xlsx
@@ -729,7 +729,7 @@
         </is>
       </c>
       <c r="B16" s="7">
-        <f>IF(NOT(ISNUMBER($B$5)),0,IF($B$5&lt;=INDEX(Piano!$A$12:$A$20,1),0,IF($B$5&gt;=INDEX(Piano!$A$12:$A$20,9),INDEX(Piano!$B$12:$B$20,9),INDEX(Piano!$B$12:$B$20,MATCH($B$5,Piano!$A$12:$A$20,1))+($B$5-INDEX(Piano!$A$12:$A$20,MATCH($B$5,Piano!$A$12:$A$20,1)))/(INDEX(Piano!$A$12:$A$20,MATCH($B$5,Piano!$A$12:$A$20,1)+1)-INDEX(Piano!$A$12:$A$20,MATCH($B$5,Piano!$A$12:$A$20,1)))*(INDEX(Piano!$B$12:$B$20,MATCH($B$5,Piano!$A$12:$A$20,1)+1)-INDEX(Piano!$B$12:$B$20,MATCH($B$5,Piano!$A$12:$A$20,1))))))</f>
+        <f>IF(NOT(ISNUMBER($B$5)),0,IF($B$5&lt;=INDEX(Piano!$A$12:$A$14,1),0,IF($B$5&gt;=INDEX(Piano!$A$12:$A$14,3),INDEX(Piano!$B$12:$B$14,3),INDEX(Piano!$B$12:$B$14,MATCH($B$5,Piano!$A$12:$A$14,1))+($B$5-INDEX(Piano!$A$12:$A$14,MATCH($B$5,Piano!$A$12:$A$14,1)))/(INDEX(Piano!$A$12:$A$14,MATCH($B$5,Piano!$A$12:$A$14,1)+1)-INDEX(Piano!$A$12:$A$14,MATCH($B$5,Piano!$A$12:$A$14,1)))*(INDEX(Piano!$B$12:$B$14,MATCH($B$5,Piano!$A$12:$A$14,1)+1)-INDEX(Piano!$B$12:$B$14,MATCH($B$5,Piano!$A$12:$A$14,1))))))</f>
         <v/>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -5916,7 +5916,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Lotta Club Seggiano — abbonamento semestrale 35×6 + quota iscrizione (previsto, ~20-30 €)</t>
+          <t>Lotta Club Seggiano — abbonamento SEMESTRALE 35×6 + quota iscrizione, una tantum: NIENTE rate mensili fino a marzo (previsto, ~20-30 €)</t>
         </is>
       </c>
       <c r="C6" s="12" t="n">
@@ -9556,7 +9556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -9626,7 +9626,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Impegni noti non ancora nel piano mensile qui sotto</t>
+          <t>Impegni noti, pagati dal conto corrente (non dal fondo)</t>
         </is>
       </c>
     </row>
@@ -9640,14 +9640,14 @@
     <row r="9">
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>• Lotta Club Seggiano: ~235 € una tantum a ottobre + 35 €/mese da novembre (previsto, vedi foglio Spese).</t>
+          <t>• Lotta Club Seggiano: ~235 € una tantum a ottobre (semestrale + quota iscrizione). Nessuna rata mensile fino a marzo 2027 — il corso è già pagato per il semestre.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>• Rimborso 730: 1.481 € netti attesi nov/dic, più preciso dei ~1.160 € stimati prima (vedi foglio Entrate).</t>
+          <t>• Rimborso 730: 1.481 € netti attesi nov/dic (vedi foglio Entrate). Non ancora nella curva sotto: la aggiungo quando arriva davvero.</t>
         </is>
       </c>
     </row>
@@ -9683,14 +9683,14 @@
     </row>
     <row r="13">
       <c r="A13" s="15" t="n">
-        <v>46295</v>
+        <v>46285</v>
       </c>
       <c r="B13" s="16" t="n">
-        <v>446</v>
+        <v>470</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>446 € versati a settembre — oggi (20/09) sei già a 470 € di fondo: leggermente avanti.</t>
+          <t>Saldo reale letto dal foglio Settimane il 20/09.</t>
         </is>
       </c>
     </row>
@@ -9699,91 +9699,35 @@
         <v>46326</v>
       </c>
       <c r="B14" s="16" t="n">
-        <v>1442</v>
+        <v>1020</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>446 + 550 € dai tuoi (affitto a 700 e 250 € da tuo padre), al netto di assicurazione e lotta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="15" t="n">
-        <v>46356</v>
-      </c>
-      <c r="B15" s="16" t="n">
-        <v>2188</v>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>446 + 300 € dai tuoi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="15" t="n">
-        <v>46387</v>
-      </c>
-      <c r="B16" s="16" t="n">
-        <v>4094</v>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>446 + 300 € dai tuoi + 1.481 € di rimborso 730 (di cui parte tenuta da parte per i regali).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="15" t="n">
-        <v>46418</v>
-      </c>
-      <c r="B17" s="16" t="n">
-        <v>4355</v>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Netto sceso a ~2.005 €: al fondo restano ~261 €/mese, da ricontrollare con la rata lotta da 35 €.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="15" t="n">
-        <v>46446</v>
-      </c>
-      <c r="B18" s="16" t="n">
-        <v>4616</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="15" t="n">
-        <v>46477</v>
-      </c>
-      <c r="B19" s="16" t="n">
-        <v>4877</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="15" t="n">
-        <v>46507</v>
-      </c>
-      <c r="B20" s="16" t="n">
-        <v>5138</v>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Traguardo raggiunto — data da confermare con i dati reali di ottobre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="40" customHeight="1">
-      <c r="A22" s="3" t="inlineStr">
+          <t>470 + 550 € versati a ottobre (deciso il 20/09). Assicurazione e lotta escono dal conto corrente, non dal fondo: non riducono questo numero.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="50" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Da novembre in poi</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Non ancora stimato: manca la conferma se il tuo stipendio netto "a regime" e i 250 € di tuo padre sono ricorrenti o solo di ottobre, e quando arriva davvero il rimborso 730. Appena hai il primo dato reale di novembre (foglio Settimane), aggiungo il punto qui invece di indovinarlo adesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Fonte dei numeri</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>Piano concordato il 13/09/2026, aggiornato il 20/09/2026 con i dati reali di assicurazione, 730 e caldaia. Questa curva mensile resta una stima: ricalcolala a fine ottobre con i numeri veri del primo mese di lotta e assicurazione pagati.</t>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Piano concordato il 13/09/2026. Curva rifatta il 20/09/2026 dopo un errore: la versione precedente non era stata ricalcolata con i costi reali di caldaia, assicurazione e lotta, e contava la lotta come rata mensile mentre è un pagamento semestrale unico.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
finanze: aggiunge la tredicesima 2026 (stima, 800 €) al foglio Entrate
</commit_message>
<xml_diff>
--- a/finanze/quaderno-5000.xlsx
+++ b/finanze/quaderno-5000.xlsx
@@ -6525,9 +6525,17 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="n"/>
-      <c r="B8" s="19" t="n"/>
-      <c r="C8" s="14" t="n"/>
+      <c r="A8" s="11" t="n">
+        <v>46357</v>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Tredicesima 2026 — 5/12 da assunzione 03/08/2026, netto stimato dal cedolino di agosto (previsto)</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>800</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="18" t="n"/>

</xml_diff>

<commit_message>
finanze: corregge il costo della lotta a 25 €/mese (non 35), 3 allenamenti/settimana
</commit_message>
<xml_diff>
--- a/finanze/quaderno-5000.xlsx
+++ b/finanze/quaderno-5000.xlsx
@@ -5916,11 +5916,11 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Lotta Club Seggiano — abbonamento SEMESTRALE 35×6 + quota iscrizione, una tantum: NIENTE rate mensili fino a marzo (previsto, ~20-30 €)</t>
+          <t>Lotta Club Seggiano — abbonamento SEMESTRALE 25×6 (corretto da 35) + quota iscrizione, una tantum: NIENTE rate mensili fino a marzo (previsto, ~20-30 €). 3 allenamenti/settimana, stesso prezzo.</t>
         </is>
       </c>
       <c r="C6" s="12" t="n">
-        <v>235</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
finanze: lotta è mensile (50€ + 25€/mese) non semestrale, stipendio confermato 2.197€
Corretto anche l'errore precedente che trattava la lotta come pagamento
semestrale una tantum: è mensile, quindi diventa un costo fisso ricorrente
da novembre, non più una spesa dal buffer. Frequenza reale: 2 volte/settimana.
</commit_message>
<xml_diff>
--- a/finanze/quaderno-5000.xlsx
+++ b/finanze/quaderno-5000.xlsx
@@ -5911,16 +5911,16 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="n">
+      <c r="A6" s="15" t="n">
         <v>46300</v>
       </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Lotta Club Seggiano — abbonamento SEMESTRALE 25×6 (corretto da 35) + quota iscrizione, una tantum: NIENTE rate mensili fino a marzo (previsto, ~20-30 €). 3 allenamenti/settimana, stesso prezzo.</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="n">
-        <v>175</v>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>Lotta Club Seggiano — quota iscrizione + primo mese, MENSILE non semestrale (corretto): dal secondo mese 25 €/mese ricorrenti, va nel budget fisso non più qui. 2 allenamenti/settimana per ora.</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="7">
@@ -6473,16 +6473,16 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="n">
-        <v>46296</v>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>Stipendio di settembre (previsto, ~2.190 €)</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="n">
-        <v>2190</v>
+      <c r="A4" s="15" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>Stipendio di settembre — accreditato, confermato</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="n">
+        <v>2197</v>
       </c>
     </row>
     <row r="5">
@@ -9648,7 +9648,7 @@
     <row r="9">
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>• Lotta Club Seggiano: ~235 € una tantum a ottobre (semestrale + quota iscrizione). Nessuna rata mensile fino a marzo 2027 — il corso è già pagato per il semestre.</t>
+          <t>• Lotta Club Seggiano: 50 € a ottobre (iscrizione + primo mese), poi 25 €/mese ricorrenti — è mensile, non semestrale (corretto). Da novembre è un costo fisso ricorrente, non più una spesa una tantum del buffer.</t>
         </is>
       </c>
     </row>

</xml_diff>